<commit_message>
Handle mixed date text formats and extend template to 800 rows
pandas' to_datetime infers one format from the first value and applies
it to the whole column, so a sheet mixing "2026-09-11" and "2026/9/10"
style dates raised instead of parsing; parse with format="mixed" and
surface unparseable dates as a per-file error like the other checks.
Also grows the pre-formatted/dropdown rows in the input template from
120 to 800 so more than a year of daily entries per store still get
the store dropdown and date formatting without manual copy-down.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155nCVn5tK4kRe72k9sPUbq
</commit_message>
<xml_diff>
--- a/dashboard/templates/日次売上_入力テンプレート.xlsx
+++ b/dashboard/templates/日次売上_入力テンプレート.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -584,6 +584,55 @@
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>・売上金額には文字や単位（円など）を含めず、数値のみを入力してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>・行の入力順序は関係ありません（新しい日付が上でも下でも、順不同でも問題なく集計されます）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>・日付は必ず「日付」として入力してください（例: 2026/9/10 や 2026-9-10 と入力すればExcelが自動で</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　日付として認識し、表示は yyyy-mm-dd になります）。「2026年9月10日」のような文字列や、</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　20260910のような数値としての入力はできません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>・過去1年以上のデータをまとめて入力しても問題ありません（前年同日比や着地予測の精度が上がります）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　あらかじめ800行分（約2年強）に書式とプルダウンを用意していますが、それを超えて入力する場合は、</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　最後の行を選択してコピーし、続きの行に貼り付ければ書式・プルダウンを引き継げます。</t>
         </is>
       </c>
     </row>
@@ -752,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1629,9 +1678,4769 @@
       <c r="D121" s="7" t="n"/>
       <c r="E121" s="5" t="n"/>
     </row>
+    <row r="122">
+      <c r="A122" s="6" t="n"/>
+      <c r="B122" s="5" t="n"/>
+      <c r="C122" s="7" t="n"/>
+      <c r="D122" s="7" t="n"/>
+      <c r="E122" s="5" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="n"/>
+      <c r="B123" s="5" t="n"/>
+      <c r="C123" s="7" t="n"/>
+      <c r="D123" s="7" t="n"/>
+      <c r="E123" s="5" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="6" t="n"/>
+      <c r="B124" s="5" t="n"/>
+      <c r="C124" s="7" t="n"/>
+      <c r="D124" s="7" t="n"/>
+      <c r="E124" s="5" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="n"/>
+      <c r="B125" s="5" t="n"/>
+      <c r="C125" s="7" t="n"/>
+      <c r="D125" s="7" t="n"/>
+      <c r="E125" s="5" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="6" t="n"/>
+      <c r="B126" s="5" t="n"/>
+      <c r="C126" s="7" t="n"/>
+      <c r="D126" s="7" t="n"/>
+      <c r="E126" s="5" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="n"/>
+      <c r="B127" s="5" t="n"/>
+      <c r="C127" s="7" t="n"/>
+      <c r="D127" s="7" t="n"/>
+      <c r="E127" s="5" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="n"/>
+      <c r="B128" s="5" t="n"/>
+      <c r="C128" s="7" t="n"/>
+      <c r="D128" s="7" t="n"/>
+      <c r="E128" s="5" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="6" t="n"/>
+      <c r="B129" s="5" t="n"/>
+      <c r="C129" s="7" t="n"/>
+      <c r="D129" s="7" t="n"/>
+      <c r="E129" s="5" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="n"/>
+      <c r="B130" s="5" t="n"/>
+      <c r="C130" s="7" t="n"/>
+      <c r="D130" s="7" t="n"/>
+      <c r="E130" s="5" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="n"/>
+      <c r="B131" s="5" t="n"/>
+      <c r="C131" s="7" t="n"/>
+      <c r="D131" s="7" t="n"/>
+      <c r="E131" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="n"/>
+      <c r="B132" s="5" t="n"/>
+      <c r="C132" s="7" t="n"/>
+      <c r="D132" s="7" t="n"/>
+      <c r="E132" s="5" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="6" t="n"/>
+      <c r="B133" s="5" t="n"/>
+      <c r="C133" s="7" t="n"/>
+      <c r="D133" s="7" t="n"/>
+      <c r="E133" s="5" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="n"/>
+      <c r="B134" s="5" t="n"/>
+      <c r="C134" s="7" t="n"/>
+      <c r="D134" s="7" t="n"/>
+      <c r="E134" s="5" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="n"/>
+      <c r="B135" s="5" t="n"/>
+      <c r="C135" s="7" t="n"/>
+      <c r="D135" s="7" t="n"/>
+      <c r="E135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="n"/>
+      <c r="B136" s="5" t="n"/>
+      <c r="C136" s="7" t="n"/>
+      <c r="D136" s="7" t="n"/>
+      <c r="E136" s="5" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="n"/>
+      <c r="B137" s="5" t="n"/>
+      <c r="C137" s="7" t="n"/>
+      <c r="D137" s="7" t="n"/>
+      <c r="E137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="n"/>
+      <c r="B138" s="5" t="n"/>
+      <c r="C138" s="7" t="n"/>
+      <c r="D138" s="7" t="n"/>
+      <c r="E138" s="5" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="6" t="n"/>
+      <c r="B139" s="5" t="n"/>
+      <c r="C139" s="7" t="n"/>
+      <c r="D139" s="7" t="n"/>
+      <c r="E139" s="5" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="n"/>
+      <c r="B140" s="5" t="n"/>
+      <c r="C140" s="7" t="n"/>
+      <c r="D140" s="7" t="n"/>
+      <c r="E140" s="5" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="n"/>
+      <c r="B141" s="5" t="n"/>
+      <c r="C141" s="7" t="n"/>
+      <c r="D141" s="7" t="n"/>
+      <c r="E141" s="5" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="n"/>
+      <c r="B142" s="5" t="n"/>
+      <c r="C142" s="7" t="n"/>
+      <c r="D142" s="7" t="n"/>
+      <c r="E142" s="5" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="n"/>
+      <c r="B143" s="5" t="n"/>
+      <c r="C143" s="7" t="n"/>
+      <c r="D143" s="7" t="n"/>
+      <c r="E143" s="5" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="n"/>
+      <c r="B144" s="5" t="n"/>
+      <c r="C144" s="7" t="n"/>
+      <c r="D144" s="7" t="n"/>
+      <c r="E144" s="5" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="n"/>
+      <c r="B145" s="5" t="n"/>
+      <c r="C145" s="7" t="n"/>
+      <c r="D145" s="7" t="n"/>
+      <c r="E145" s="5" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="n"/>
+      <c r="B146" s="5" t="n"/>
+      <c r="C146" s="7" t="n"/>
+      <c r="D146" s="7" t="n"/>
+      <c r="E146" s="5" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="n"/>
+      <c r="B147" s="5" t="n"/>
+      <c r="C147" s="7" t="n"/>
+      <c r="D147" s="7" t="n"/>
+      <c r="E147" s="5" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="n"/>
+      <c r="B148" s="5" t="n"/>
+      <c r="C148" s="7" t="n"/>
+      <c r="D148" s="7" t="n"/>
+      <c r="E148" s="5" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="6" t="n"/>
+      <c r="B149" s="5" t="n"/>
+      <c r="C149" s="7" t="n"/>
+      <c r="D149" s="7" t="n"/>
+      <c r="E149" s="5" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="6" t="n"/>
+      <c r="B150" s="5" t="n"/>
+      <c r="C150" s="7" t="n"/>
+      <c r="D150" s="7" t="n"/>
+      <c r="E150" s="5" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="n"/>
+      <c r="B151" s="5" t="n"/>
+      <c r="C151" s="7" t="n"/>
+      <c r="D151" s="7" t="n"/>
+      <c r="E151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="6" t="n"/>
+      <c r="B152" s="5" t="n"/>
+      <c r="C152" s="7" t="n"/>
+      <c r="D152" s="7" t="n"/>
+      <c r="E152" s="5" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="6" t="n"/>
+      <c r="B153" s="5" t="n"/>
+      <c r="C153" s="7" t="n"/>
+      <c r="D153" s="7" t="n"/>
+      <c r="E153" s="5" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="6" t="n"/>
+      <c r="B154" s="5" t="n"/>
+      <c r="C154" s="7" t="n"/>
+      <c r="D154" s="7" t="n"/>
+      <c r="E154" s="5" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="6" t="n"/>
+      <c r="B155" s="5" t="n"/>
+      <c r="C155" s="7" t="n"/>
+      <c r="D155" s="7" t="n"/>
+      <c r="E155" s="5" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="n"/>
+      <c r="B156" s="5" t="n"/>
+      <c r="C156" s="7" t="n"/>
+      <c r="D156" s="7" t="n"/>
+      <c r="E156" s="5" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="n"/>
+      <c r="B157" s="5" t="n"/>
+      <c r="C157" s="7" t="n"/>
+      <c r="D157" s="7" t="n"/>
+      <c r="E157" s="5" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="n"/>
+      <c r="B158" s="5" t="n"/>
+      <c r="C158" s="7" t="n"/>
+      <c r="D158" s="7" t="n"/>
+      <c r="E158" s="5" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="n"/>
+      <c r="B159" s="5" t="n"/>
+      <c r="C159" s="7" t="n"/>
+      <c r="D159" s="7" t="n"/>
+      <c r="E159" s="5" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="n"/>
+      <c r="B160" s="5" t="n"/>
+      <c r="C160" s="7" t="n"/>
+      <c r="D160" s="7" t="n"/>
+      <c r="E160" s="5" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="6" t="n"/>
+      <c r="B161" s="5" t="n"/>
+      <c r="C161" s="7" t="n"/>
+      <c r="D161" s="7" t="n"/>
+      <c r="E161" s="5" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="n"/>
+      <c r="B162" s="5" t="n"/>
+      <c r="C162" s="7" t="n"/>
+      <c r="D162" s="7" t="n"/>
+      <c r="E162" s="5" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="6" t="n"/>
+      <c r="B163" s="5" t="n"/>
+      <c r="C163" s="7" t="n"/>
+      <c r="D163" s="7" t="n"/>
+      <c r="E163" s="5" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="6" t="n"/>
+      <c r="B164" s="5" t="n"/>
+      <c r="C164" s="7" t="n"/>
+      <c r="D164" s="7" t="n"/>
+      <c r="E164" s="5" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="n"/>
+      <c r="B165" s="5" t="n"/>
+      <c r="C165" s="7" t="n"/>
+      <c r="D165" s="7" t="n"/>
+      <c r="E165" s="5" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="6" t="n"/>
+      <c r="B166" s="5" t="n"/>
+      <c r="C166" s="7" t="n"/>
+      <c r="D166" s="7" t="n"/>
+      <c r="E166" s="5" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="n"/>
+      <c r="B167" s="5" t="n"/>
+      <c r="C167" s="7" t="n"/>
+      <c r="D167" s="7" t="n"/>
+      <c r="E167" s="5" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="6" t="n"/>
+      <c r="B168" s="5" t="n"/>
+      <c r="C168" s="7" t="n"/>
+      <c r="D168" s="7" t="n"/>
+      <c r="E168" s="5" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="6" t="n"/>
+      <c r="B169" s="5" t="n"/>
+      <c r="C169" s="7" t="n"/>
+      <c r="D169" s="7" t="n"/>
+      <c r="E169" s="5" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="6" t="n"/>
+      <c r="B170" s="5" t="n"/>
+      <c r="C170" s="7" t="n"/>
+      <c r="D170" s="7" t="n"/>
+      <c r="E170" s="5" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="6" t="n"/>
+      <c r="B171" s="5" t="n"/>
+      <c r="C171" s="7" t="n"/>
+      <c r="D171" s="7" t="n"/>
+      <c r="E171" s="5" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="6" t="n"/>
+      <c r="B172" s="5" t="n"/>
+      <c r="C172" s="7" t="n"/>
+      <c r="D172" s="7" t="n"/>
+      <c r="E172" s="5" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="n"/>
+      <c r="B173" s="5" t="n"/>
+      <c r="C173" s="7" t="n"/>
+      <c r="D173" s="7" t="n"/>
+      <c r="E173" s="5" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="6" t="n"/>
+      <c r="B174" s="5" t="n"/>
+      <c r="C174" s="7" t="n"/>
+      <c r="D174" s="7" t="n"/>
+      <c r="E174" s="5" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="n"/>
+      <c r="B175" s="5" t="n"/>
+      <c r="C175" s="7" t="n"/>
+      <c r="D175" s="7" t="n"/>
+      <c r="E175" s="5" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="n"/>
+      <c r="B176" s="5" t="n"/>
+      <c r="C176" s="7" t="n"/>
+      <c r="D176" s="7" t="n"/>
+      <c r="E176" s="5" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="6" t="n"/>
+      <c r="B177" s="5" t="n"/>
+      <c r="C177" s="7" t="n"/>
+      <c r="D177" s="7" t="n"/>
+      <c r="E177" s="5" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="6" t="n"/>
+      <c r="B178" s="5" t="n"/>
+      <c r="C178" s="7" t="n"/>
+      <c r="D178" s="7" t="n"/>
+      <c r="E178" s="5" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="6" t="n"/>
+      <c r="B179" s="5" t="n"/>
+      <c r="C179" s="7" t="n"/>
+      <c r="D179" s="7" t="n"/>
+      <c r="E179" s="5" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="6" t="n"/>
+      <c r="B180" s="5" t="n"/>
+      <c r="C180" s="7" t="n"/>
+      <c r="D180" s="7" t="n"/>
+      <c r="E180" s="5" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="6" t="n"/>
+      <c r="B181" s="5" t="n"/>
+      <c r="C181" s="7" t="n"/>
+      <c r="D181" s="7" t="n"/>
+      <c r="E181" s="5" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="6" t="n"/>
+      <c r="B182" s="5" t="n"/>
+      <c r="C182" s="7" t="n"/>
+      <c r="D182" s="7" t="n"/>
+      <c r="E182" s="5" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="6" t="n"/>
+      <c r="B183" s="5" t="n"/>
+      <c r="C183" s="7" t="n"/>
+      <c r="D183" s="7" t="n"/>
+      <c r="E183" s="5" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="6" t="n"/>
+      <c r="B184" s="5" t="n"/>
+      <c r="C184" s="7" t="n"/>
+      <c r="D184" s="7" t="n"/>
+      <c r="E184" s="5" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="6" t="n"/>
+      <c r="B185" s="5" t="n"/>
+      <c r="C185" s="7" t="n"/>
+      <c r="D185" s="7" t="n"/>
+      <c r="E185" s="5" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="6" t="n"/>
+      <c r="B186" s="5" t="n"/>
+      <c r="C186" s="7" t="n"/>
+      <c r="D186" s="7" t="n"/>
+      <c r="E186" s="5" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="6" t="n"/>
+      <c r="B187" s="5" t="n"/>
+      <c r="C187" s="7" t="n"/>
+      <c r="D187" s="7" t="n"/>
+      <c r="E187" s="5" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="6" t="n"/>
+      <c r="B188" s="5" t="n"/>
+      <c r="C188" s="7" t="n"/>
+      <c r="D188" s="7" t="n"/>
+      <c r="E188" s="5" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="6" t="n"/>
+      <c r="B189" s="5" t="n"/>
+      <c r="C189" s="7" t="n"/>
+      <c r="D189" s="7" t="n"/>
+      <c r="E189" s="5" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="6" t="n"/>
+      <c r="B190" s="5" t="n"/>
+      <c r="C190" s="7" t="n"/>
+      <c r="D190" s="7" t="n"/>
+      <c r="E190" s="5" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="6" t="n"/>
+      <c r="B191" s="5" t="n"/>
+      <c r="C191" s="7" t="n"/>
+      <c r="D191" s="7" t="n"/>
+      <c r="E191" s="5" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="6" t="n"/>
+      <c r="B192" s="5" t="n"/>
+      <c r="C192" s="7" t="n"/>
+      <c r="D192" s="7" t="n"/>
+      <c r="E192" s="5" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="6" t="n"/>
+      <c r="B193" s="5" t="n"/>
+      <c r="C193" s="7" t="n"/>
+      <c r="D193" s="7" t="n"/>
+      <c r="E193" s="5" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="6" t="n"/>
+      <c r="B194" s="5" t="n"/>
+      <c r="C194" s="7" t="n"/>
+      <c r="D194" s="7" t="n"/>
+      <c r="E194" s="5" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="6" t="n"/>
+      <c r="B195" s="5" t="n"/>
+      <c r="C195" s="7" t="n"/>
+      <c r="D195" s="7" t="n"/>
+      <c r="E195" s="5" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="6" t="n"/>
+      <c r="B196" s="5" t="n"/>
+      <c r="C196" s="7" t="n"/>
+      <c r="D196" s="7" t="n"/>
+      <c r="E196" s="5" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="6" t="n"/>
+      <c r="B197" s="5" t="n"/>
+      <c r="C197" s="7" t="n"/>
+      <c r="D197" s="7" t="n"/>
+      <c r="E197" s="5" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="6" t="n"/>
+      <c r="B198" s="5" t="n"/>
+      <c r="C198" s="7" t="n"/>
+      <c r="D198" s="7" t="n"/>
+      <c r="E198" s="5" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="6" t="n"/>
+      <c r="B199" s="5" t="n"/>
+      <c r="C199" s="7" t="n"/>
+      <c r="D199" s="7" t="n"/>
+      <c r="E199" s="5" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="6" t="n"/>
+      <c r="B200" s="5" t="n"/>
+      <c r="C200" s="7" t="n"/>
+      <c r="D200" s="7" t="n"/>
+      <c r="E200" s="5" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="6" t="n"/>
+      <c r="B201" s="5" t="n"/>
+      <c r="C201" s="7" t="n"/>
+      <c r="D201" s="7" t="n"/>
+      <c r="E201" s="5" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="6" t="n"/>
+      <c r="B202" s="5" t="n"/>
+      <c r="C202" s="7" t="n"/>
+      <c r="D202" s="7" t="n"/>
+      <c r="E202" s="5" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="6" t="n"/>
+      <c r="B203" s="5" t="n"/>
+      <c r="C203" s="7" t="n"/>
+      <c r="D203" s="7" t="n"/>
+      <c r="E203" s="5" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="6" t="n"/>
+      <c r="B204" s="5" t="n"/>
+      <c r="C204" s="7" t="n"/>
+      <c r="D204" s="7" t="n"/>
+      <c r="E204" s="5" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="6" t="n"/>
+      <c r="B205" s="5" t="n"/>
+      <c r="C205" s="7" t="n"/>
+      <c r="D205" s="7" t="n"/>
+      <c r="E205" s="5" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="6" t="n"/>
+      <c r="B206" s="5" t="n"/>
+      <c r="C206" s="7" t="n"/>
+      <c r="D206" s="7" t="n"/>
+      <c r="E206" s="5" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="6" t="n"/>
+      <c r="B207" s="5" t="n"/>
+      <c r="C207" s="7" t="n"/>
+      <c r="D207" s="7" t="n"/>
+      <c r="E207" s="5" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="6" t="n"/>
+      <c r="B208" s="5" t="n"/>
+      <c r="C208" s="7" t="n"/>
+      <c r="D208" s="7" t="n"/>
+      <c r="E208" s="5" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="6" t="n"/>
+      <c r="B209" s="5" t="n"/>
+      <c r="C209" s="7" t="n"/>
+      <c r="D209" s="7" t="n"/>
+      <c r="E209" s="5" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="6" t="n"/>
+      <c r="B210" s="5" t="n"/>
+      <c r="C210" s="7" t="n"/>
+      <c r="D210" s="7" t="n"/>
+      <c r="E210" s="5" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="6" t="n"/>
+      <c r="B211" s="5" t="n"/>
+      <c r="C211" s="7" t="n"/>
+      <c r="D211" s="7" t="n"/>
+      <c r="E211" s="5" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="6" t="n"/>
+      <c r="B212" s="5" t="n"/>
+      <c r="C212" s="7" t="n"/>
+      <c r="D212" s="7" t="n"/>
+      <c r="E212" s="5" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="6" t="n"/>
+      <c r="B213" s="5" t="n"/>
+      <c r="C213" s="7" t="n"/>
+      <c r="D213" s="7" t="n"/>
+      <c r="E213" s="5" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="6" t="n"/>
+      <c r="B214" s="5" t="n"/>
+      <c r="C214" s="7" t="n"/>
+      <c r="D214" s="7" t="n"/>
+      <c r="E214" s="5" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="6" t="n"/>
+      <c r="B215" s="5" t="n"/>
+      <c r="C215" s="7" t="n"/>
+      <c r="D215" s="7" t="n"/>
+      <c r="E215" s="5" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="6" t="n"/>
+      <c r="B216" s="5" t="n"/>
+      <c r="C216" s="7" t="n"/>
+      <c r="D216" s="7" t="n"/>
+      <c r="E216" s="5" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="6" t="n"/>
+      <c r="B217" s="5" t="n"/>
+      <c r="C217" s="7" t="n"/>
+      <c r="D217" s="7" t="n"/>
+      <c r="E217" s="5" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="6" t="n"/>
+      <c r="B218" s="5" t="n"/>
+      <c r="C218" s="7" t="n"/>
+      <c r="D218" s="7" t="n"/>
+      <c r="E218" s="5" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="6" t="n"/>
+      <c r="B219" s="5" t="n"/>
+      <c r="C219" s="7" t="n"/>
+      <c r="D219" s="7" t="n"/>
+      <c r="E219" s="5" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="6" t="n"/>
+      <c r="B220" s="5" t="n"/>
+      <c r="C220" s="7" t="n"/>
+      <c r="D220" s="7" t="n"/>
+      <c r="E220" s="5" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="6" t="n"/>
+      <c r="B221" s="5" t="n"/>
+      <c r="C221" s="7" t="n"/>
+      <c r="D221" s="7" t="n"/>
+      <c r="E221" s="5" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="6" t="n"/>
+      <c r="B222" s="5" t="n"/>
+      <c r="C222" s="7" t="n"/>
+      <c r="D222" s="7" t="n"/>
+      <c r="E222" s="5" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="6" t="n"/>
+      <c r="B223" s="5" t="n"/>
+      <c r="C223" s="7" t="n"/>
+      <c r="D223" s="7" t="n"/>
+      <c r="E223" s="5" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="6" t="n"/>
+      <c r="B224" s="5" t="n"/>
+      <c r="C224" s="7" t="n"/>
+      <c r="D224" s="7" t="n"/>
+      <c r="E224" s="5" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="6" t="n"/>
+      <c r="B225" s="5" t="n"/>
+      <c r="C225" s="7" t="n"/>
+      <c r="D225" s="7" t="n"/>
+      <c r="E225" s="5" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="6" t="n"/>
+      <c r="B226" s="5" t="n"/>
+      <c r="C226" s="7" t="n"/>
+      <c r="D226" s="7" t="n"/>
+      <c r="E226" s="5" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="6" t="n"/>
+      <c r="B227" s="5" t="n"/>
+      <c r="C227" s="7" t="n"/>
+      <c r="D227" s="7" t="n"/>
+      <c r="E227" s="5" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="6" t="n"/>
+      <c r="B228" s="5" t="n"/>
+      <c r="C228" s="7" t="n"/>
+      <c r="D228" s="7" t="n"/>
+      <c r="E228" s="5" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="6" t="n"/>
+      <c r="B229" s="5" t="n"/>
+      <c r="C229" s="7" t="n"/>
+      <c r="D229" s="7" t="n"/>
+      <c r="E229" s="5" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="6" t="n"/>
+      <c r="B230" s="5" t="n"/>
+      <c r="C230" s="7" t="n"/>
+      <c r="D230" s="7" t="n"/>
+      <c r="E230" s="5" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="6" t="n"/>
+      <c r="B231" s="5" t="n"/>
+      <c r="C231" s="7" t="n"/>
+      <c r="D231" s="7" t="n"/>
+      <c r="E231" s="5" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="6" t="n"/>
+      <c r="B232" s="5" t="n"/>
+      <c r="C232" s="7" t="n"/>
+      <c r="D232" s="7" t="n"/>
+      <c r="E232" s="5" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="6" t="n"/>
+      <c r="B233" s="5" t="n"/>
+      <c r="C233" s="7" t="n"/>
+      <c r="D233" s="7" t="n"/>
+      <c r="E233" s="5" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="6" t="n"/>
+      <c r="B234" s="5" t="n"/>
+      <c r="C234" s="7" t="n"/>
+      <c r="D234" s="7" t="n"/>
+      <c r="E234" s="5" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="6" t="n"/>
+      <c r="B235" s="5" t="n"/>
+      <c r="C235" s="7" t="n"/>
+      <c r="D235" s="7" t="n"/>
+      <c r="E235" s="5" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="6" t="n"/>
+      <c r="B236" s="5" t="n"/>
+      <c r="C236" s="7" t="n"/>
+      <c r="D236" s="7" t="n"/>
+      <c r="E236" s="5" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="6" t="n"/>
+      <c r="B237" s="5" t="n"/>
+      <c r="C237" s="7" t="n"/>
+      <c r="D237" s="7" t="n"/>
+      <c r="E237" s="5" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="6" t="n"/>
+      <c r="B238" s="5" t="n"/>
+      <c r="C238" s="7" t="n"/>
+      <c r="D238" s="7" t="n"/>
+      <c r="E238" s="5" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="6" t="n"/>
+      <c r="B239" s="5" t="n"/>
+      <c r="C239" s="7" t="n"/>
+      <c r="D239" s="7" t="n"/>
+      <c r="E239" s="5" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="6" t="n"/>
+      <c r="B240" s="5" t="n"/>
+      <c r="C240" s="7" t="n"/>
+      <c r="D240" s="7" t="n"/>
+      <c r="E240" s="5" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="6" t="n"/>
+      <c r="B241" s="5" t="n"/>
+      <c r="C241" s="7" t="n"/>
+      <c r="D241" s="7" t="n"/>
+      <c r="E241" s="5" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="6" t="n"/>
+      <c r="B242" s="5" t="n"/>
+      <c r="C242" s="7" t="n"/>
+      <c r="D242" s="7" t="n"/>
+      <c r="E242" s="5" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="6" t="n"/>
+      <c r="B243" s="5" t="n"/>
+      <c r="C243" s="7" t="n"/>
+      <c r="D243" s="7" t="n"/>
+      <c r="E243" s="5" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="6" t="n"/>
+      <c r="B244" s="5" t="n"/>
+      <c r="C244" s="7" t="n"/>
+      <c r="D244" s="7" t="n"/>
+      <c r="E244" s="5" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="6" t="n"/>
+      <c r="B245" s="5" t="n"/>
+      <c r="C245" s="7" t="n"/>
+      <c r="D245" s="7" t="n"/>
+      <c r="E245" s="5" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="6" t="n"/>
+      <c r="B246" s="5" t="n"/>
+      <c r="C246" s="7" t="n"/>
+      <c r="D246" s="7" t="n"/>
+      <c r="E246" s="5" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="6" t="n"/>
+      <c r="B247" s="5" t="n"/>
+      <c r="C247" s="7" t="n"/>
+      <c r="D247" s="7" t="n"/>
+      <c r="E247" s="5" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="6" t="n"/>
+      <c r="B248" s="5" t="n"/>
+      <c r="C248" s="7" t="n"/>
+      <c r="D248" s="7" t="n"/>
+      <c r="E248" s="5" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="6" t="n"/>
+      <c r="B249" s="5" t="n"/>
+      <c r="C249" s="7" t="n"/>
+      <c r="D249" s="7" t="n"/>
+      <c r="E249" s="5" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="6" t="n"/>
+      <c r="B250" s="5" t="n"/>
+      <c r="C250" s="7" t="n"/>
+      <c r="D250" s="7" t="n"/>
+      <c r="E250" s="5" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="6" t="n"/>
+      <c r="B251" s="5" t="n"/>
+      <c r="C251" s="7" t="n"/>
+      <c r="D251" s="7" t="n"/>
+      <c r="E251" s="5" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="6" t="n"/>
+      <c r="B252" s="5" t="n"/>
+      <c r="C252" s="7" t="n"/>
+      <c r="D252" s="7" t="n"/>
+      <c r="E252" s="5" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="6" t="n"/>
+      <c r="B253" s="5" t="n"/>
+      <c r="C253" s="7" t="n"/>
+      <c r="D253" s="7" t="n"/>
+      <c r="E253" s="5" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="6" t="n"/>
+      <c r="B254" s="5" t="n"/>
+      <c r="C254" s="7" t="n"/>
+      <c r="D254" s="7" t="n"/>
+      <c r="E254" s="5" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="6" t="n"/>
+      <c r="B255" s="5" t="n"/>
+      <c r="C255" s="7" t="n"/>
+      <c r="D255" s="7" t="n"/>
+      <c r="E255" s="5" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="6" t="n"/>
+      <c r="B256" s="5" t="n"/>
+      <c r="C256" s="7" t="n"/>
+      <c r="D256" s="7" t="n"/>
+      <c r="E256" s="5" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="6" t="n"/>
+      <c r="B257" s="5" t="n"/>
+      <c r="C257" s="7" t="n"/>
+      <c r="D257" s="7" t="n"/>
+      <c r="E257" s="5" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="6" t="n"/>
+      <c r="B258" s="5" t="n"/>
+      <c r="C258" s="7" t="n"/>
+      <c r="D258" s="7" t="n"/>
+      <c r="E258" s="5" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="6" t="n"/>
+      <c r="B259" s="5" t="n"/>
+      <c r="C259" s="7" t="n"/>
+      <c r="D259" s="7" t="n"/>
+      <c r="E259" s="5" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="6" t="n"/>
+      <c r="B260" s="5" t="n"/>
+      <c r="C260" s="7" t="n"/>
+      <c r="D260" s="7" t="n"/>
+      <c r="E260" s="5" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="6" t="n"/>
+      <c r="B261" s="5" t="n"/>
+      <c r="C261" s="7" t="n"/>
+      <c r="D261" s="7" t="n"/>
+      <c r="E261" s="5" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="6" t="n"/>
+      <c r="B262" s="5" t="n"/>
+      <c r="C262" s="7" t="n"/>
+      <c r="D262" s="7" t="n"/>
+      <c r="E262" s="5" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="6" t="n"/>
+      <c r="B263" s="5" t="n"/>
+      <c r="C263" s="7" t="n"/>
+      <c r="D263" s="7" t="n"/>
+      <c r="E263" s="5" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="6" t="n"/>
+      <c r="B264" s="5" t="n"/>
+      <c r="C264" s="7" t="n"/>
+      <c r="D264" s="7" t="n"/>
+      <c r="E264" s="5" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="6" t="n"/>
+      <c r="B265" s="5" t="n"/>
+      <c r="C265" s="7" t="n"/>
+      <c r="D265" s="7" t="n"/>
+      <c r="E265" s="5" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="6" t="n"/>
+      <c r="B266" s="5" t="n"/>
+      <c r="C266" s="7" t="n"/>
+      <c r="D266" s="7" t="n"/>
+      <c r="E266" s="5" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="6" t="n"/>
+      <c r="B267" s="5" t="n"/>
+      <c r="C267" s="7" t="n"/>
+      <c r="D267" s="7" t="n"/>
+      <c r="E267" s="5" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="6" t="n"/>
+      <c r="B268" s="5" t="n"/>
+      <c r="C268" s="7" t="n"/>
+      <c r="D268" s="7" t="n"/>
+      <c r="E268" s="5" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="6" t="n"/>
+      <c r="B269" s="5" t="n"/>
+      <c r="C269" s="7" t="n"/>
+      <c r="D269" s="7" t="n"/>
+      <c r="E269" s="5" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="6" t="n"/>
+      <c r="B270" s="5" t="n"/>
+      <c r="C270" s="7" t="n"/>
+      <c r="D270" s="7" t="n"/>
+      <c r="E270" s="5" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="6" t="n"/>
+      <c r="B271" s="5" t="n"/>
+      <c r="C271" s="7" t="n"/>
+      <c r="D271" s="7" t="n"/>
+      <c r="E271" s="5" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="6" t="n"/>
+      <c r="B272" s="5" t="n"/>
+      <c r="C272" s="7" t="n"/>
+      <c r="D272" s="7" t="n"/>
+      <c r="E272" s="5" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="6" t="n"/>
+      <c r="B273" s="5" t="n"/>
+      <c r="C273" s="7" t="n"/>
+      <c r="D273" s="7" t="n"/>
+      <c r="E273" s="5" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="6" t="n"/>
+      <c r="B274" s="5" t="n"/>
+      <c r="C274" s="7" t="n"/>
+      <c r="D274" s="7" t="n"/>
+      <c r="E274" s="5" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="6" t="n"/>
+      <c r="B275" s="5" t="n"/>
+      <c r="C275" s="7" t="n"/>
+      <c r="D275" s="7" t="n"/>
+      <c r="E275" s="5" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="6" t="n"/>
+      <c r="B276" s="5" t="n"/>
+      <c r="C276" s="7" t="n"/>
+      <c r="D276" s="7" t="n"/>
+      <c r="E276" s="5" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="6" t="n"/>
+      <c r="B277" s="5" t="n"/>
+      <c r="C277" s="7" t="n"/>
+      <c r="D277" s="7" t="n"/>
+      <c r="E277" s="5" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="6" t="n"/>
+      <c r="B278" s="5" t="n"/>
+      <c r="C278" s="7" t="n"/>
+      <c r="D278" s="7" t="n"/>
+      <c r="E278" s="5" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="6" t="n"/>
+      <c r="B279" s="5" t="n"/>
+      <c r="C279" s="7" t="n"/>
+      <c r="D279" s="7" t="n"/>
+      <c r="E279" s="5" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="6" t="n"/>
+      <c r="B280" s="5" t="n"/>
+      <c r="C280" s="7" t="n"/>
+      <c r="D280" s="7" t="n"/>
+      <c r="E280" s="5" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="6" t="n"/>
+      <c r="B281" s="5" t="n"/>
+      <c r="C281" s="7" t="n"/>
+      <c r="D281" s="7" t="n"/>
+      <c r="E281" s="5" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="6" t="n"/>
+      <c r="B282" s="5" t="n"/>
+      <c r="C282" s="7" t="n"/>
+      <c r="D282" s="7" t="n"/>
+      <c r="E282" s="5" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="6" t="n"/>
+      <c r="B283" s="5" t="n"/>
+      <c r="C283" s="7" t="n"/>
+      <c r="D283" s="7" t="n"/>
+      <c r="E283" s="5" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="6" t="n"/>
+      <c r="B284" s="5" t="n"/>
+      <c r="C284" s="7" t="n"/>
+      <c r="D284" s="7" t="n"/>
+      <c r="E284" s="5" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="6" t="n"/>
+      <c r="B285" s="5" t="n"/>
+      <c r="C285" s="7" t="n"/>
+      <c r="D285" s="7" t="n"/>
+      <c r="E285" s="5" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="6" t="n"/>
+      <c r="B286" s="5" t="n"/>
+      <c r="C286" s="7" t="n"/>
+      <c r="D286" s="7" t="n"/>
+      <c r="E286" s="5" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="6" t="n"/>
+      <c r="B287" s="5" t="n"/>
+      <c r="C287" s="7" t="n"/>
+      <c r="D287" s="7" t="n"/>
+      <c r="E287" s="5" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="6" t="n"/>
+      <c r="B288" s="5" t="n"/>
+      <c r="C288" s="7" t="n"/>
+      <c r="D288" s="7" t="n"/>
+      <c r="E288" s="5" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="6" t="n"/>
+      <c r="B289" s="5" t="n"/>
+      <c r="C289" s="7" t="n"/>
+      <c r="D289" s="7" t="n"/>
+      <c r="E289" s="5" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="6" t="n"/>
+      <c r="B290" s="5" t="n"/>
+      <c r="C290" s="7" t="n"/>
+      <c r="D290" s="7" t="n"/>
+      <c r="E290" s="5" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="6" t="n"/>
+      <c r="B291" s="5" t="n"/>
+      <c r="C291" s="7" t="n"/>
+      <c r="D291" s="7" t="n"/>
+      <c r="E291" s="5" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="6" t="n"/>
+      <c r="B292" s="5" t="n"/>
+      <c r="C292" s="7" t="n"/>
+      <c r="D292" s="7" t="n"/>
+      <c r="E292" s="5" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="6" t="n"/>
+      <c r="B293" s="5" t="n"/>
+      <c r="C293" s="7" t="n"/>
+      <c r="D293" s="7" t="n"/>
+      <c r="E293" s="5" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="6" t="n"/>
+      <c r="B294" s="5" t="n"/>
+      <c r="C294" s="7" t="n"/>
+      <c r="D294" s="7" t="n"/>
+      <c r="E294" s="5" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="6" t="n"/>
+      <c r="B295" s="5" t="n"/>
+      <c r="C295" s="7" t="n"/>
+      <c r="D295" s="7" t="n"/>
+      <c r="E295" s="5" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="6" t="n"/>
+      <c r="B296" s="5" t="n"/>
+      <c r="C296" s="7" t="n"/>
+      <c r="D296" s="7" t="n"/>
+      <c r="E296" s="5" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="6" t="n"/>
+      <c r="B297" s="5" t="n"/>
+      <c r="C297" s="7" t="n"/>
+      <c r="D297" s="7" t="n"/>
+      <c r="E297" s="5" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="6" t="n"/>
+      <c r="B298" s="5" t="n"/>
+      <c r="C298" s="7" t="n"/>
+      <c r="D298" s="7" t="n"/>
+      <c r="E298" s="5" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="6" t="n"/>
+      <c r="B299" s="5" t="n"/>
+      <c r="C299" s="7" t="n"/>
+      <c r="D299" s="7" t="n"/>
+      <c r="E299" s="5" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="6" t="n"/>
+      <c r="B300" s="5" t="n"/>
+      <c r="C300" s="7" t="n"/>
+      <c r="D300" s="7" t="n"/>
+      <c r="E300" s="5" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="6" t="n"/>
+      <c r="B301" s="5" t="n"/>
+      <c r="C301" s="7" t="n"/>
+      <c r="D301" s="7" t="n"/>
+      <c r="E301" s="5" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="6" t="n"/>
+      <c r="B302" s="5" t="n"/>
+      <c r="C302" s="7" t="n"/>
+      <c r="D302" s="7" t="n"/>
+      <c r="E302" s="5" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="6" t="n"/>
+      <c r="B303" s="5" t="n"/>
+      <c r="C303" s="7" t="n"/>
+      <c r="D303" s="7" t="n"/>
+      <c r="E303" s="5" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="6" t="n"/>
+      <c r="B304" s="5" t="n"/>
+      <c r="C304" s="7" t="n"/>
+      <c r="D304" s="7" t="n"/>
+      <c r="E304" s="5" t="n"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="6" t="n"/>
+      <c r="B305" s="5" t="n"/>
+      <c r="C305" s="7" t="n"/>
+      <c r="D305" s="7" t="n"/>
+      <c r="E305" s="5" t="n"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="6" t="n"/>
+      <c r="B306" s="5" t="n"/>
+      <c r="C306" s="7" t="n"/>
+      <c r="D306" s="7" t="n"/>
+      <c r="E306" s="5" t="n"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="6" t="n"/>
+      <c r="B307" s="5" t="n"/>
+      <c r="C307" s="7" t="n"/>
+      <c r="D307" s="7" t="n"/>
+      <c r="E307" s="5" t="n"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="6" t="n"/>
+      <c r="B308" s="5" t="n"/>
+      <c r="C308" s="7" t="n"/>
+      <c r="D308" s="7" t="n"/>
+      <c r="E308" s="5" t="n"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="6" t="n"/>
+      <c r="B309" s="5" t="n"/>
+      <c r="C309" s="7" t="n"/>
+      <c r="D309" s="7" t="n"/>
+      <c r="E309" s="5" t="n"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="6" t="n"/>
+      <c r="B310" s="5" t="n"/>
+      <c r="C310" s="7" t="n"/>
+      <c r="D310" s="7" t="n"/>
+      <c r="E310" s="5" t="n"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="6" t="n"/>
+      <c r="B311" s="5" t="n"/>
+      <c r="C311" s="7" t="n"/>
+      <c r="D311" s="7" t="n"/>
+      <c r="E311" s="5" t="n"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="6" t="n"/>
+      <c r="B312" s="5" t="n"/>
+      <c r="C312" s="7" t="n"/>
+      <c r="D312" s="7" t="n"/>
+      <c r="E312" s="5" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="6" t="n"/>
+      <c r="B313" s="5" t="n"/>
+      <c r="C313" s="7" t="n"/>
+      <c r="D313" s="7" t="n"/>
+      <c r="E313" s="5" t="n"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="6" t="n"/>
+      <c r="B314" s="5" t="n"/>
+      <c r="C314" s="7" t="n"/>
+      <c r="D314" s="7" t="n"/>
+      <c r="E314" s="5" t="n"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="6" t="n"/>
+      <c r="B315" s="5" t="n"/>
+      <c r="C315" s="7" t="n"/>
+      <c r="D315" s="7" t="n"/>
+      <c r="E315" s="5" t="n"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="6" t="n"/>
+      <c r="B316" s="5" t="n"/>
+      <c r="C316" s="7" t="n"/>
+      <c r="D316" s="7" t="n"/>
+      <c r="E316" s="5" t="n"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="6" t="n"/>
+      <c r="B317" s="5" t="n"/>
+      <c r="C317" s="7" t="n"/>
+      <c r="D317" s="7" t="n"/>
+      <c r="E317" s="5" t="n"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="6" t="n"/>
+      <c r="B318" s="5" t="n"/>
+      <c r="C318" s="7" t="n"/>
+      <c r="D318" s="7" t="n"/>
+      <c r="E318" s="5" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="6" t="n"/>
+      <c r="B319" s="5" t="n"/>
+      <c r="C319" s="7" t="n"/>
+      <c r="D319" s="7" t="n"/>
+      <c r="E319" s="5" t="n"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="6" t="n"/>
+      <c r="B320" s="5" t="n"/>
+      <c r="C320" s="7" t="n"/>
+      <c r="D320" s="7" t="n"/>
+      <c r="E320" s="5" t="n"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="6" t="n"/>
+      <c r="B321" s="5" t="n"/>
+      <c r="C321" s="7" t="n"/>
+      <c r="D321" s="7" t="n"/>
+      <c r="E321" s="5" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="6" t="n"/>
+      <c r="B322" s="5" t="n"/>
+      <c r="C322" s="7" t="n"/>
+      <c r="D322" s="7" t="n"/>
+      <c r="E322" s="5" t="n"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="6" t="n"/>
+      <c r="B323" s="5" t="n"/>
+      <c r="C323" s="7" t="n"/>
+      <c r="D323" s="7" t="n"/>
+      <c r="E323" s="5" t="n"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="6" t="n"/>
+      <c r="B324" s="5" t="n"/>
+      <c r="C324" s="7" t="n"/>
+      <c r="D324" s="7" t="n"/>
+      <c r="E324" s="5" t="n"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="6" t="n"/>
+      <c r="B325" s="5" t="n"/>
+      <c r="C325" s="7" t="n"/>
+      <c r="D325" s="7" t="n"/>
+      <c r="E325" s="5" t="n"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="6" t="n"/>
+      <c r="B326" s="5" t="n"/>
+      <c r="C326" s="7" t="n"/>
+      <c r="D326" s="7" t="n"/>
+      <c r="E326" s="5" t="n"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="6" t="n"/>
+      <c r="B327" s="5" t="n"/>
+      <c r="C327" s="7" t="n"/>
+      <c r="D327" s="7" t="n"/>
+      <c r="E327" s="5" t="n"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="6" t="n"/>
+      <c r="B328" s="5" t="n"/>
+      <c r="C328" s="7" t="n"/>
+      <c r="D328" s="7" t="n"/>
+      <c r="E328" s="5" t="n"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="6" t="n"/>
+      <c r="B329" s="5" t="n"/>
+      <c r="C329" s="7" t="n"/>
+      <c r="D329" s="7" t="n"/>
+      <c r="E329" s="5" t="n"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="6" t="n"/>
+      <c r="B330" s="5" t="n"/>
+      <c r="C330" s="7" t="n"/>
+      <c r="D330" s="7" t="n"/>
+      <c r="E330" s="5" t="n"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="6" t="n"/>
+      <c r="B331" s="5" t="n"/>
+      <c r="C331" s="7" t="n"/>
+      <c r="D331" s="7" t="n"/>
+      <c r="E331" s="5" t="n"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="6" t="n"/>
+      <c r="B332" s="5" t="n"/>
+      <c r="C332" s="7" t="n"/>
+      <c r="D332" s="7" t="n"/>
+      <c r="E332" s="5" t="n"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="6" t="n"/>
+      <c r="B333" s="5" t="n"/>
+      <c r="C333" s="7" t="n"/>
+      <c r="D333" s="7" t="n"/>
+      <c r="E333" s="5" t="n"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="6" t="n"/>
+      <c r="B334" s="5" t="n"/>
+      <c r="C334" s="7" t="n"/>
+      <c r="D334" s="7" t="n"/>
+      <c r="E334" s="5" t="n"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="6" t="n"/>
+      <c r="B335" s="5" t="n"/>
+      <c r="C335" s="7" t="n"/>
+      <c r="D335" s="7" t="n"/>
+      <c r="E335" s="5" t="n"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="6" t="n"/>
+      <c r="B336" s="5" t="n"/>
+      <c r="C336" s="7" t="n"/>
+      <c r="D336" s="7" t="n"/>
+      <c r="E336" s="5" t="n"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="6" t="n"/>
+      <c r="B337" s="5" t="n"/>
+      <c r="C337" s="7" t="n"/>
+      <c r="D337" s="7" t="n"/>
+      <c r="E337" s="5" t="n"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="6" t="n"/>
+      <c r="B338" s="5" t="n"/>
+      <c r="C338" s="7" t="n"/>
+      <c r="D338" s="7" t="n"/>
+      <c r="E338" s="5" t="n"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="6" t="n"/>
+      <c r="B339" s="5" t="n"/>
+      <c r="C339" s="7" t="n"/>
+      <c r="D339" s="7" t="n"/>
+      <c r="E339" s="5" t="n"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="6" t="n"/>
+      <c r="B340" s="5" t="n"/>
+      <c r="C340" s="7" t="n"/>
+      <c r="D340" s="7" t="n"/>
+      <c r="E340" s="5" t="n"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="6" t="n"/>
+      <c r="B341" s="5" t="n"/>
+      <c r="C341" s="7" t="n"/>
+      <c r="D341" s="7" t="n"/>
+      <c r="E341" s="5" t="n"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="6" t="n"/>
+      <c r="B342" s="5" t="n"/>
+      <c r="C342" s="7" t="n"/>
+      <c r="D342" s="7" t="n"/>
+      <c r="E342" s="5" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="6" t="n"/>
+      <c r="B343" s="5" t="n"/>
+      <c r="C343" s="7" t="n"/>
+      <c r="D343" s="7" t="n"/>
+      <c r="E343" s="5" t="n"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="6" t="n"/>
+      <c r="B344" s="5" t="n"/>
+      <c r="C344" s="7" t="n"/>
+      <c r="D344" s="7" t="n"/>
+      <c r="E344" s="5" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="6" t="n"/>
+      <c r="B345" s="5" t="n"/>
+      <c r="C345" s="7" t="n"/>
+      <c r="D345" s="7" t="n"/>
+      <c r="E345" s="5" t="n"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="6" t="n"/>
+      <c r="B346" s="5" t="n"/>
+      <c r="C346" s="7" t="n"/>
+      <c r="D346" s="7" t="n"/>
+      <c r="E346" s="5" t="n"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="6" t="n"/>
+      <c r="B347" s="5" t="n"/>
+      <c r="C347" s="7" t="n"/>
+      <c r="D347" s="7" t="n"/>
+      <c r="E347" s="5" t="n"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="6" t="n"/>
+      <c r="B348" s="5" t="n"/>
+      <c r="C348" s="7" t="n"/>
+      <c r="D348" s="7" t="n"/>
+      <c r="E348" s="5" t="n"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="6" t="n"/>
+      <c r="B349" s="5" t="n"/>
+      <c r="C349" s="7" t="n"/>
+      <c r="D349" s="7" t="n"/>
+      <c r="E349" s="5" t="n"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="6" t="n"/>
+      <c r="B350" s="5" t="n"/>
+      <c r="C350" s="7" t="n"/>
+      <c r="D350" s="7" t="n"/>
+      <c r="E350" s="5" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="6" t="n"/>
+      <c r="B351" s="5" t="n"/>
+      <c r="C351" s="7" t="n"/>
+      <c r="D351" s="7" t="n"/>
+      <c r="E351" s="5" t="n"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="6" t="n"/>
+      <c r="B352" s="5" t="n"/>
+      <c r="C352" s="7" t="n"/>
+      <c r="D352" s="7" t="n"/>
+      <c r="E352" s="5" t="n"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="6" t="n"/>
+      <c r="B353" s="5" t="n"/>
+      <c r="C353" s="7" t="n"/>
+      <c r="D353" s="7" t="n"/>
+      <c r="E353" s="5" t="n"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="6" t="n"/>
+      <c r="B354" s="5" t="n"/>
+      <c r="C354" s="7" t="n"/>
+      <c r="D354" s="7" t="n"/>
+      <c r="E354" s="5" t="n"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="6" t="n"/>
+      <c r="B355" s="5" t="n"/>
+      <c r="C355" s="7" t="n"/>
+      <c r="D355" s="7" t="n"/>
+      <c r="E355" s="5" t="n"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="6" t="n"/>
+      <c r="B356" s="5" t="n"/>
+      <c r="C356" s="7" t="n"/>
+      <c r="D356" s="7" t="n"/>
+      <c r="E356" s="5" t="n"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="6" t="n"/>
+      <c r="B357" s="5" t="n"/>
+      <c r="C357" s="7" t="n"/>
+      <c r="D357" s="7" t="n"/>
+      <c r="E357" s="5" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="6" t="n"/>
+      <c r="B358" s="5" t="n"/>
+      <c r="C358" s="7" t="n"/>
+      <c r="D358" s="7" t="n"/>
+      <c r="E358" s="5" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="6" t="n"/>
+      <c r="B359" s="5" t="n"/>
+      <c r="C359" s="7" t="n"/>
+      <c r="D359" s="7" t="n"/>
+      <c r="E359" s="5" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="6" t="n"/>
+      <c r="B360" s="5" t="n"/>
+      <c r="C360" s="7" t="n"/>
+      <c r="D360" s="7" t="n"/>
+      <c r="E360" s="5" t="n"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="6" t="n"/>
+      <c r="B361" s="5" t="n"/>
+      <c r="C361" s="7" t="n"/>
+      <c r="D361" s="7" t="n"/>
+      <c r="E361" s="5" t="n"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="6" t="n"/>
+      <c r="B362" s="5" t="n"/>
+      <c r="C362" s="7" t="n"/>
+      <c r="D362" s="7" t="n"/>
+      <c r="E362" s="5" t="n"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="6" t="n"/>
+      <c r="B363" s="5" t="n"/>
+      <c r="C363" s="7" t="n"/>
+      <c r="D363" s="7" t="n"/>
+      <c r="E363" s="5" t="n"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="6" t="n"/>
+      <c r="B364" s="5" t="n"/>
+      <c r="C364" s="7" t="n"/>
+      <c r="D364" s="7" t="n"/>
+      <c r="E364" s="5" t="n"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="6" t="n"/>
+      <c r="B365" s="5" t="n"/>
+      <c r="C365" s="7" t="n"/>
+      <c r="D365" s="7" t="n"/>
+      <c r="E365" s="5" t="n"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="6" t="n"/>
+      <c r="B366" s="5" t="n"/>
+      <c r="C366" s="7" t="n"/>
+      <c r="D366" s="7" t="n"/>
+      <c r="E366" s="5" t="n"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="6" t="n"/>
+      <c r="B367" s="5" t="n"/>
+      <c r="C367" s="7" t="n"/>
+      <c r="D367" s="7" t="n"/>
+      <c r="E367" s="5" t="n"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="6" t="n"/>
+      <c r="B368" s="5" t="n"/>
+      <c r="C368" s="7" t="n"/>
+      <c r="D368" s="7" t="n"/>
+      <c r="E368" s="5" t="n"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="6" t="n"/>
+      <c r="B369" s="5" t="n"/>
+      <c r="C369" s="7" t="n"/>
+      <c r="D369" s="7" t="n"/>
+      <c r="E369" s="5" t="n"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="6" t="n"/>
+      <c r="B370" s="5" t="n"/>
+      <c r="C370" s="7" t="n"/>
+      <c r="D370" s="7" t="n"/>
+      <c r="E370" s="5" t="n"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="6" t="n"/>
+      <c r="B371" s="5" t="n"/>
+      <c r="C371" s="7" t="n"/>
+      <c r="D371" s="7" t="n"/>
+      <c r="E371" s="5" t="n"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="6" t="n"/>
+      <c r="B372" s="5" t="n"/>
+      <c r="C372" s="7" t="n"/>
+      <c r="D372" s="7" t="n"/>
+      <c r="E372" s="5" t="n"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="6" t="n"/>
+      <c r="B373" s="5" t="n"/>
+      <c r="C373" s="7" t="n"/>
+      <c r="D373" s="7" t="n"/>
+      <c r="E373" s="5" t="n"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="6" t="n"/>
+      <c r="B374" s="5" t="n"/>
+      <c r="C374" s="7" t="n"/>
+      <c r="D374" s="7" t="n"/>
+      <c r="E374" s="5" t="n"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="6" t="n"/>
+      <c r="B375" s="5" t="n"/>
+      <c r="C375" s="7" t="n"/>
+      <c r="D375" s="7" t="n"/>
+      <c r="E375" s="5" t="n"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="6" t="n"/>
+      <c r="B376" s="5" t="n"/>
+      <c r="C376" s="7" t="n"/>
+      <c r="D376" s="7" t="n"/>
+      <c r="E376" s="5" t="n"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="6" t="n"/>
+      <c r="B377" s="5" t="n"/>
+      <c r="C377" s="7" t="n"/>
+      <c r="D377" s="7" t="n"/>
+      <c r="E377" s="5" t="n"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="6" t="n"/>
+      <c r="B378" s="5" t="n"/>
+      <c r="C378" s="7" t="n"/>
+      <c r="D378" s="7" t="n"/>
+      <c r="E378" s="5" t="n"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="6" t="n"/>
+      <c r="B379" s="5" t="n"/>
+      <c r="C379" s="7" t="n"/>
+      <c r="D379" s="7" t="n"/>
+      <c r="E379" s="5" t="n"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="6" t="n"/>
+      <c r="B380" s="5" t="n"/>
+      <c r="C380" s="7" t="n"/>
+      <c r="D380" s="7" t="n"/>
+      <c r="E380" s="5" t="n"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="6" t="n"/>
+      <c r="B381" s="5" t="n"/>
+      <c r="C381" s="7" t="n"/>
+      <c r="D381" s="7" t="n"/>
+      <c r="E381" s="5" t="n"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="6" t="n"/>
+      <c r="B382" s="5" t="n"/>
+      <c r="C382" s="7" t="n"/>
+      <c r="D382" s="7" t="n"/>
+      <c r="E382" s="5" t="n"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="6" t="n"/>
+      <c r="B383" s="5" t="n"/>
+      <c r="C383" s="7" t="n"/>
+      <c r="D383" s="7" t="n"/>
+      <c r="E383" s="5" t="n"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="6" t="n"/>
+      <c r="B384" s="5" t="n"/>
+      <c r="C384" s="7" t="n"/>
+      <c r="D384" s="7" t="n"/>
+      <c r="E384" s="5" t="n"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="6" t="n"/>
+      <c r="B385" s="5" t="n"/>
+      <c r="C385" s="7" t="n"/>
+      <c r="D385" s="7" t="n"/>
+      <c r="E385" s="5" t="n"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="6" t="n"/>
+      <c r="B386" s="5" t="n"/>
+      <c r="C386" s="7" t="n"/>
+      <c r="D386" s="7" t="n"/>
+      <c r="E386" s="5" t="n"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="6" t="n"/>
+      <c r="B387" s="5" t="n"/>
+      <c r="C387" s="7" t="n"/>
+      <c r="D387" s="7" t="n"/>
+      <c r="E387" s="5" t="n"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="6" t="n"/>
+      <c r="B388" s="5" t="n"/>
+      <c r="C388" s="7" t="n"/>
+      <c r="D388" s="7" t="n"/>
+      <c r="E388" s="5" t="n"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="6" t="n"/>
+      <c r="B389" s="5" t="n"/>
+      <c r="C389" s="7" t="n"/>
+      <c r="D389" s="7" t="n"/>
+      <c r="E389" s="5" t="n"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="6" t="n"/>
+      <c r="B390" s="5" t="n"/>
+      <c r="C390" s="7" t="n"/>
+      <c r="D390" s="7" t="n"/>
+      <c r="E390" s="5" t="n"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="6" t="n"/>
+      <c r="B391" s="5" t="n"/>
+      <c r="C391" s="7" t="n"/>
+      <c r="D391" s="7" t="n"/>
+      <c r="E391" s="5" t="n"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="6" t="n"/>
+      <c r="B392" s="5" t="n"/>
+      <c r="C392" s="7" t="n"/>
+      <c r="D392" s="7" t="n"/>
+      <c r="E392" s="5" t="n"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="6" t="n"/>
+      <c r="B393" s="5" t="n"/>
+      <c r="C393" s="7" t="n"/>
+      <c r="D393" s="7" t="n"/>
+      <c r="E393" s="5" t="n"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="6" t="n"/>
+      <c r="B394" s="5" t="n"/>
+      <c r="C394" s="7" t="n"/>
+      <c r="D394" s="7" t="n"/>
+      <c r="E394" s="5" t="n"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="6" t="n"/>
+      <c r="B395" s="5" t="n"/>
+      <c r="C395" s="7" t="n"/>
+      <c r="D395" s="7" t="n"/>
+      <c r="E395" s="5" t="n"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="6" t="n"/>
+      <c r="B396" s="5" t="n"/>
+      <c r="C396" s="7" t="n"/>
+      <c r="D396" s="7" t="n"/>
+      <c r="E396" s="5" t="n"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="6" t="n"/>
+      <c r="B397" s="5" t="n"/>
+      <c r="C397" s="7" t="n"/>
+      <c r="D397" s="7" t="n"/>
+      <c r="E397" s="5" t="n"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="6" t="n"/>
+      <c r="B398" s="5" t="n"/>
+      <c r="C398" s="7" t="n"/>
+      <c r="D398" s="7" t="n"/>
+      <c r="E398" s="5" t="n"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="6" t="n"/>
+      <c r="B399" s="5" t="n"/>
+      <c r="C399" s="7" t="n"/>
+      <c r="D399" s="7" t="n"/>
+      <c r="E399" s="5" t="n"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="6" t="n"/>
+      <c r="B400" s="5" t="n"/>
+      <c r="C400" s="7" t="n"/>
+      <c r="D400" s="7" t="n"/>
+      <c r="E400" s="5" t="n"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="6" t="n"/>
+      <c r="B401" s="5" t="n"/>
+      <c r="C401" s="7" t="n"/>
+      <c r="D401" s="7" t="n"/>
+      <c r="E401" s="5" t="n"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="6" t="n"/>
+      <c r="B402" s="5" t="n"/>
+      <c r="C402" s="7" t="n"/>
+      <c r="D402" s="7" t="n"/>
+      <c r="E402" s="5" t="n"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="6" t="n"/>
+      <c r="B403" s="5" t="n"/>
+      <c r="C403" s="7" t="n"/>
+      <c r="D403" s="7" t="n"/>
+      <c r="E403" s="5" t="n"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="6" t="n"/>
+      <c r="B404" s="5" t="n"/>
+      <c r="C404" s="7" t="n"/>
+      <c r="D404" s="7" t="n"/>
+      <c r="E404" s="5" t="n"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="6" t="n"/>
+      <c r="B405" s="5" t="n"/>
+      <c r="C405" s="7" t="n"/>
+      <c r="D405" s="7" t="n"/>
+      <c r="E405" s="5" t="n"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="6" t="n"/>
+      <c r="B406" s="5" t="n"/>
+      <c r="C406" s="7" t="n"/>
+      <c r="D406" s="7" t="n"/>
+      <c r="E406" s="5" t="n"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="6" t="n"/>
+      <c r="B407" s="5" t="n"/>
+      <c r="C407" s="7" t="n"/>
+      <c r="D407" s="7" t="n"/>
+      <c r="E407" s="5" t="n"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="6" t="n"/>
+      <c r="B408" s="5" t="n"/>
+      <c r="C408" s="7" t="n"/>
+      <c r="D408" s="7" t="n"/>
+      <c r="E408" s="5" t="n"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="6" t="n"/>
+      <c r="B409" s="5" t="n"/>
+      <c r="C409" s="7" t="n"/>
+      <c r="D409" s="7" t="n"/>
+      <c r="E409" s="5" t="n"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="6" t="n"/>
+      <c r="B410" s="5" t="n"/>
+      <c r="C410" s="7" t="n"/>
+      <c r="D410" s="7" t="n"/>
+      <c r="E410" s="5" t="n"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="6" t="n"/>
+      <c r="B411" s="5" t="n"/>
+      <c r="C411" s="7" t="n"/>
+      <c r="D411" s="7" t="n"/>
+      <c r="E411" s="5" t="n"/>
+    </row>
+    <row r="412">
+      <c r="A412" s="6" t="n"/>
+      <c r="B412" s="5" t="n"/>
+      <c r="C412" s="7" t="n"/>
+      <c r="D412" s="7" t="n"/>
+      <c r="E412" s="5" t="n"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="6" t="n"/>
+      <c r="B413" s="5" t="n"/>
+      <c r="C413" s="7" t="n"/>
+      <c r="D413" s="7" t="n"/>
+      <c r="E413" s="5" t="n"/>
+    </row>
+    <row r="414">
+      <c r="A414" s="6" t="n"/>
+      <c r="B414" s="5" t="n"/>
+      <c r="C414" s="7" t="n"/>
+      <c r="D414" s="7" t="n"/>
+      <c r="E414" s="5" t="n"/>
+    </row>
+    <row r="415">
+      <c r="A415" s="6" t="n"/>
+      <c r="B415" s="5" t="n"/>
+      <c r="C415" s="7" t="n"/>
+      <c r="D415" s="7" t="n"/>
+      <c r="E415" s="5" t="n"/>
+    </row>
+    <row r="416">
+      <c r="A416" s="6" t="n"/>
+      <c r="B416" s="5" t="n"/>
+      <c r="C416" s="7" t="n"/>
+      <c r="D416" s="7" t="n"/>
+      <c r="E416" s="5" t="n"/>
+    </row>
+    <row r="417">
+      <c r="A417" s="6" t="n"/>
+      <c r="B417" s="5" t="n"/>
+      <c r="C417" s="7" t="n"/>
+      <c r="D417" s="7" t="n"/>
+      <c r="E417" s="5" t="n"/>
+    </row>
+    <row r="418">
+      <c r="A418" s="6" t="n"/>
+      <c r="B418" s="5" t="n"/>
+      <c r="C418" s="7" t="n"/>
+      <c r="D418" s="7" t="n"/>
+      <c r="E418" s="5" t="n"/>
+    </row>
+    <row r="419">
+      <c r="A419" s="6" t="n"/>
+      <c r="B419" s="5" t="n"/>
+      <c r="C419" s="7" t="n"/>
+      <c r="D419" s="7" t="n"/>
+      <c r="E419" s="5" t="n"/>
+    </row>
+    <row r="420">
+      <c r="A420" s="6" t="n"/>
+      <c r="B420" s="5" t="n"/>
+      <c r="C420" s="7" t="n"/>
+      <c r="D420" s="7" t="n"/>
+      <c r="E420" s="5" t="n"/>
+    </row>
+    <row r="421">
+      <c r="A421" s="6" t="n"/>
+      <c r="B421" s="5" t="n"/>
+      <c r="C421" s="7" t="n"/>
+      <c r="D421" s="7" t="n"/>
+      <c r="E421" s="5" t="n"/>
+    </row>
+    <row r="422">
+      <c r="A422" s="6" t="n"/>
+      <c r="B422" s="5" t="n"/>
+      <c r="C422" s="7" t="n"/>
+      <c r="D422" s="7" t="n"/>
+      <c r="E422" s="5" t="n"/>
+    </row>
+    <row r="423">
+      <c r="A423" s="6" t="n"/>
+      <c r="B423" s="5" t="n"/>
+      <c r="C423" s="7" t="n"/>
+      <c r="D423" s="7" t="n"/>
+      <c r="E423" s="5" t="n"/>
+    </row>
+    <row r="424">
+      <c r="A424" s="6" t="n"/>
+      <c r="B424" s="5" t="n"/>
+      <c r="C424" s="7" t="n"/>
+      <c r="D424" s="7" t="n"/>
+      <c r="E424" s="5" t="n"/>
+    </row>
+    <row r="425">
+      <c r="A425" s="6" t="n"/>
+      <c r="B425" s="5" t="n"/>
+      <c r="C425" s="7" t="n"/>
+      <c r="D425" s="7" t="n"/>
+      <c r="E425" s="5" t="n"/>
+    </row>
+    <row r="426">
+      <c r="A426" s="6" t="n"/>
+      <c r="B426" s="5" t="n"/>
+      <c r="C426" s="7" t="n"/>
+      <c r="D426" s="7" t="n"/>
+      <c r="E426" s="5" t="n"/>
+    </row>
+    <row r="427">
+      <c r="A427" s="6" t="n"/>
+      <c r="B427" s="5" t="n"/>
+      <c r="C427" s="7" t="n"/>
+      <c r="D427" s="7" t="n"/>
+      <c r="E427" s="5" t="n"/>
+    </row>
+    <row r="428">
+      <c r="A428" s="6" t="n"/>
+      <c r="B428" s="5" t="n"/>
+      <c r="C428" s="7" t="n"/>
+      <c r="D428" s="7" t="n"/>
+      <c r="E428" s="5" t="n"/>
+    </row>
+    <row r="429">
+      <c r="A429" s="6" t="n"/>
+      <c r="B429" s="5" t="n"/>
+      <c r="C429" s="7" t="n"/>
+      <c r="D429" s="7" t="n"/>
+      <c r="E429" s="5" t="n"/>
+    </row>
+    <row r="430">
+      <c r="A430" s="6" t="n"/>
+      <c r="B430" s="5" t="n"/>
+      <c r="C430" s="7" t="n"/>
+      <c r="D430" s="7" t="n"/>
+      <c r="E430" s="5" t="n"/>
+    </row>
+    <row r="431">
+      <c r="A431" s="6" t="n"/>
+      <c r="B431" s="5" t="n"/>
+      <c r="C431" s="7" t="n"/>
+      <c r="D431" s="7" t="n"/>
+      <c r="E431" s="5" t="n"/>
+    </row>
+    <row r="432">
+      <c r="A432" s="6" t="n"/>
+      <c r="B432" s="5" t="n"/>
+      <c r="C432" s="7" t="n"/>
+      <c r="D432" s="7" t="n"/>
+      <c r="E432" s="5" t="n"/>
+    </row>
+    <row r="433">
+      <c r="A433" s="6" t="n"/>
+      <c r="B433" s="5" t="n"/>
+      <c r="C433" s="7" t="n"/>
+      <c r="D433" s="7" t="n"/>
+      <c r="E433" s="5" t="n"/>
+    </row>
+    <row r="434">
+      <c r="A434" s="6" t="n"/>
+      <c r="B434" s="5" t="n"/>
+      <c r="C434" s="7" t="n"/>
+      <c r="D434" s="7" t="n"/>
+      <c r="E434" s="5" t="n"/>
+    </row>
+    <row r="435">
+      <c r="A435" s="6" t="n"/>
+      <c r="B435" s="5" t="n"/>
+      <c r="C435" s="7" t="n"/>
+      <c r="D435" s="7" t="n"/>
+      <c r="E435" s="5" t="n"/>
+    </row>
+    <row r="436">
+      <c r="A436" s="6" t="n"/>
+      <c r="B436" s="5" t="n"/>
+      <c r="C436" s="7" t="n"/>
+      <c r="D436" s="7" t="n"/>
+      <c r="E436" s="5" t="n"/>
+    </row>
+    <row r="437">
+      <c r="A437" s="6" t="n"/>
+      <c r="B437" s="5" t="n"/>
+      <c r="C437" s="7" t="n"/>
+      <c r="D437" s="7" t="n"/>
+      <c r="E437" s="5" t="n"/>
+    </row>
+    <row r="438">
+      <c r="A438" s="6" t="n"/>
+      <c r="B438" s="5" t="n"/>
+      <c r="C438" s="7" t="n"/>
+      <c r="D438" s="7" t="n"/>
+      <c r="E438" s="5" t="n"/>
+    </row>
+    <row r="439">
+      <c r="A439" s="6" t="n"/>
+      <c r="B439" s="5" t="n"/>
+      <c r="C439" s="7" t="n"/>
+      <c r="D439" s="7" t="n"/>
+      <c r="E439" s="5" t="n"/>
+    </row>
+    <row r="440">
+      <c r="A440" s="6" t="n"/>
+      <c r="B440" s="5" t="n"/>
+      <c r="C440" s="7" t="n"/>
+      <c r="D440" s="7" t="n"/>
+      <c r="E440" s="5" t="n"/>
+    </row>
+    <row r="441">
+      <c r="A441" s="6" t="n"/>
+      <c r="B441" s="5" t="n"/>
+      <c r="C441" s="7" t="n"/>
+      <c r="D441" s="7" t="n"/>
+      <c r="E441" s="5" t="n"/>
+    </row>
+    <row r="442">
+      <c r="A442" s="6" t="n"/>
+      <c r="B442" s="5" t="n"/>
+      <c r="C442" s="7" t="n"/>
+      <c r="D442" s="7" t="n"/>
+      <c r="E442" s="5" t="n"/>
+    </row>
+    <row r="443">
+      <c r="A443" s="6" t="n"/>
+      <c r="B443" s="5" t="n"/>
+      <c r="C443" s="7" t="n"/>
+      <c r="D443" s="7" t="n"/>
+      <c r="E443" s="5" t="n"/>
+    </row>
+    <row r="444">
+      <c r="A444" s="6" t="n"/>
+      <c r="B444" s="5" t="n"/>
+      <c r="C444" s="7" t="n"/>
+      <c r="D444" s="7" t="n"/>
+      <c r="E444" s="5" t="n"/>
+    </row>
+    <row r="445">
+      <c r="A445" s="6" t="n"/>
+      <c r="B445" s="5" t="n"/>
+      <c r="C445" s="7" t="n"/>
+      <c r="D445" s="7" t="n"/>
+      <c r="E445" s="5" t="n"/>
+    </row>
+    <row r="446">
+      <c r="A446" s="6" t="n"/>
+      <c r="B446" s="5" t="n"/>
+      <c r="C446" s="7" t="n"/>
+      <c r="D446" s="7" t="n"/>
+      <c r="E446" s="5" t="n"/>
+    </row>
+    <row r="447">
+      <c r="A447" s="6" t="n"/>
+      <c r="B447" s="5" t="n"/>
+      <c r="C447" s="7" t="n"/>
+      <c r="D447" s="7" t="n"/>
+      <c r="E447" s="5" t="n"/>
+    </row>
+    <row r="448">
+      <c r="A448" s="6" t="n"/>
+      <c r="B448" s="5" t="n"/>
+      <c r="C448" s="7" t="n"/>
+      <c r="D448" s="7" t="n"/>
+      <c r="E448" s="5" t="n"/>
+    </row>
+    <row r="449">
+      <c r="A449" s="6" t="n"/>
+      <c r="B449" s="5" t="n"/>
+      <c r="C449" s="7" t="n"/>
+      <c r="D449" s="7" t="n"/>
+      <c r="E449" s="5" t="n"/>
+    </row>
+    <row r="450">
+      <c r="A450" s="6" t="n"/>
+      <c r="B450" s="5" t="n"/>
+      <c r="C450" s="7" t="n"/>
+      <c r="D450" s="7" t="n"/>
+      <c r="E450" s="5" t="n"/>
+    </row>
+    <row r="451">
+      <c r="A451" s="6" t="n"/>
+      <c r="B451" s="5" t="n"/>
+      <c r="C451" s="7" t="n"/>
+      <c r="D451" s="7" t="n"/>
+      <c r="E451" s="5" t="n"/>
+    </row>
+    <row r="452">
+      <c r="A452" s="6" t="n"/>
+      <c r="B452" s="5" t="n"/>
+      <c r="C452" s="7" t="n"/>
+      <c r="D452" s="7" t="n"/>
+      <c r="E452" s="5" t="n"/>
+    </row>
+    <row r="453">
+      <c r="A453" s="6" t="n"/>
+      <c r="B453" s="5" t="n"/>
+      <c r="C453" s="7" t="n"/>
+      <c r="D453" s="7" t="n"/>
+      <c r="E453" s="5" t="n"/>
+    </row>
+    <row r="454">
+      <c r="A454" s="6" t="n"/>
+      <c r="B454" s="5" t="n"/>
+      <c r="C454" s="7" t="n"/>
+      <c r="D454" s="7" t="n"/>
+      <c r="E454" s="5" t="n"/>
+    </row>
+    <row r="455">
+      <c r="A455" s="6" t="n"/>
+      <c r="B455" s="5" t="n"/>
+      <c r="C455" s="7" t="n"/>
+      <c r="D455" s="7" t="n"/>
+      <c r="E455" s="5" t="n"/>
+    </row>
+    <row r="456">
+      <c r="A456" s="6" t="n"/>
+      <c r="B456" s="5" t="n"/>
+      <c r="C456" s="7" t="n"/>
+      <c r="D456" s="7" t="n"/>
+      <c r="E456" s="5" t="n"/>
+    </row>
+    <row r="457">
+      <c r="A457" s="6" t="n"/>
+      <c r="B457" s="5" t="n"/>
+      <c r="C457" s="7" t="n"/>
+      <c r="D457" s="7" t="n"/>
+      <c r="E457" s="5" t="n"/>
+    </row>
+    <row r="458">
+      <c r="A458" s="6" t="n"/>
+      <c r="B458" s="5" t="n"/>
+      <c r="C458" s="7" t="n"/>
+      <c r="D458" s="7" t="n"/>
+      <c r="E458" s="5" t="n"/>
+    </row>
+    <row r="459">
+      <c r="A459" s="6" t="n"/>
+      <c r="B459" s="5" t="n"/>
+      <c r="C459" s="7" t="n"/>
+      <c r="D459" s="7" t="n"/>
+      <c r="E459" s="5" t="n"/>
+    </row>
+    <row r="460">
+      <c r="A460" s="6" t="n"/>
+      <c r="B460" s="5" t="n"/>
+      <c r="C460" s="7" t="n"/>
+      <c r="D460" s="7" t="n"/>
+      <c r="E460" s="5" t="n"/>
+    </row>
+    <row r="461">
+      <c r="A461" s="6" t="n"/>
+      <c r="B461" s="5" t="n"/>
+      <c r="C461" s="7" t="n"/>
+      <c r="D461" s="7" t="n"/>
+      <c r="E461" s="5" t="n"/>
+    </row>
+    <row r="462">
+      <c r="A462" s="6" t="n"/>
+      <c r="B462" s="5" t="n"/>
+      <c r="C462" s="7" t="n"/>
+      <c r="D462" s="7" t="n"/>
+      <c r="E462" s="5" t="n"/>
+    </row>
+    <row r="463">
+      <c r="A463" s="6" t="n"/>
+      <c r="B463" s="5" t="n"/>
+      <c r="C463" s="7" t="n"/>
+      <c r="D463" s="7" t="n"/>
+      <c r="E463" s="5" t="n"/>
+    </row>
+    <row r="464">
+      <c r="A464" s="6" t="n"/>
+      <c r="B464" s="5" t="n"/>
+      <c r="C464" s="7" t="n"/>
+      <c r="D464" s="7" t="n"/>
+      <c r="E464" s="5" t="n"/>
+    </row>
+    <row r="465">
+      <c r="A465" s="6" t="n"/>
+      <c r="B465" s="5" t="n"/>
+      <c r="C465" s="7" t="n"/>
+      <c r="D465" s="7" t="n"/>
+      <c r="E465" s="5" t="n"/>
+    </row>
+    <row r="466">
+      <c r="A466" s="6" t="n"/>
+      <c r="B466" s="5" t="n"/>
+      <c r="C466" s="7" t="n"/>
+      <c r="D466" s="7" t="n"/>
+      <c r="E466" s="5" t="n"/>
+    </row>
+    <row r="467">
+      <c r="A467" s="6" t="n"/>
+      <c r="B467" s="5" t="n"/>
+      <c r="C467" s="7" t="n"/>
+      <c r="D467" s="7" t="n"/>
+      <c r="E467" s="5" t="n"/>
+    </row>
+    <row r="468">
+      <c r="A468" s="6" t="n"/>
+      <c r="B468" s="5" t="n"/>
+      <c r="C468" s="7" t="n"/>
+      <c r="D468" s="7" t="n"/>
+      <c r="E468" s="5" t="n"/>
+    </row>
+    <row r="469">
+      <c r="A469" s="6" t="n"/>
+      <c r="B469" s="5" t="n"/>
+      <c r="C469" s="7" t="n"/>
+      <c r="D469" s="7" t="n"/>
+      <c r="E469" s="5" t="n"/>
+    </row>
+    <row r="470">
+      <c r="A470" s="6" t="n"/>
+      <c r="B470" s="5" t="n"/>
+      <c r="C470" s="7" t="n"/>
+      <c r="D470" s="7" t="n"/>
+      <c r="E470" s="5" t="n"/>
+    </row>
+    <row r="471">
+      <c r="A471" s="6" t="n"/>
+      <c r="B471" s="5" t="n"/>
+      <c r="C471" s="7" t="n"/>
+      <c r="D471" s="7" t="n"/>
+      <c r="E471" s="5" t="n"/>
+    </row>
+    <row r="472">
+      <c r="A472" s="6" t="n"/>
+      <c r="B472" s="5" t="n"/>
+      <c r="C472" s="7" t="n"/>
+      <c r="D472" s="7" t="n"/>
+      <c r="E472" s="5" t="n"/>
+    </row>
+    <row r="473">
+      <c r="A473" s="6" t="n"/>
+      <c r="B473" s="5" t="n"/>
+      <c r="C473" s="7" t="n"/>
+      <c r="D473" s="7" t="n"/>
+      <c r="E473" s="5" t="n"/>
+    </row>
+    <row r="474">
+      <c r="A474" s="6" t="n"/>
+      <c r="B474" s="5" t="n"/>
+      <c r="C474" s="7" t="n"/>
+      <c r="D474" s="7" t="n"/>
+      <c r="E474" s="5" t="n"/>
+    </row>
+    <row r="475">
+      <c r="A475" s="6" t="n"/>
+      <c r="B475" s="5" t="n"/>
+      <c r="C475" s="7" t="n"/>
+      <c r="D475" s="7" t="n"/>
+      <c r="E475" s="5" t="n"/>
+    </row>
+    <row r="476">
+      <c r="A476" s="6" t="n"/>
+      <c r="B476" s="5" t="n"/>
+      <c r="C476" s="7" t="n"/>
+      <c r="D476" s="7" t="n"/>
+      <c r="E476" s="5" t="n"/>
+    </row>
+    <row r="477">
+      <c r="A477" s="6" t="n"/>
+      <c r="B477" s="5" t="n"/>
+      <c r="C477" s="7" t="n"/>
+      <c r="D477" s="7" t="n"/>
+      <c r="E477" s="5" t="n"/>
+    </row>
+    <row r="478">
+      <c r="A478" s="6" t="n"/>
+      <c r="B478" s="5" t="n"/>
+      <c r="C478" s="7" t="n"/>
+      <c r="D478" s="7" t="n"/>
+      <c r="E478" s="5" t="n"/>
+    </row>
+    <row r="479">
+      <c r="A479" s="6" t="n"/>
+      <c r="B479" s="5" t="n"/>
+      <c r="C479" s="7" t="n"/>
+      <c r="D479" s="7" t="n"/>
+      <c r="E479" s="5" t="n"/>
+    </row>
+    <row r="480">
+      <c r="A480" s="6" t="n"/>
+      <c r="B480" s="5" t="n"/>
+      <c r="C480" s="7" t="n"/>
+      <c r="D480" s="7" t="n"/>
+      <c r="E480" s="5" t="n"/>
+    </row>
+    <row r="481">
+      <c r="A481" s="6" t="n"/>
+      <c r="B481" s="5" t="n"/>
+      <c r="C481" s="7" t="n"/>
+      <c r="D481" s="7" t="n"/>
+      <c r="E481" s="5" t="n"/>
+    </row>
+    <row r="482">
+      <c r="A482" s="6" t="n"/>
+      <c r="B482" s="5" t="n"/>
+      <c r="C482" s="7" t="n"/>
+      <c r="D482" s="7" t="n"/>
+      <c r="E482" s="5" t="n"/>
+    </row>
+    <row r="483">
+      <c r="A483" s="6" t="n"/>
+      <c r="B483" s="5" t="n"/>
+      <c r="C483" s="7" t="n"/>
+      <c r="D483" s="7" t="n"/>
+      <c r="E483" s="5" t="n"/>
+    </row>
+    <row r="484">
+      <c r="A484" s="6" t="n"/>
+      <c r="B484" s="5" t="n"/>
+      <c r="C484" s="7" t="n"/>
+      <c r="D484" s="7" t="n"/>
+      <c r="E484" s="5" t="n"/>
+    </row>
+    <row r="485">
+      <c r="A485" s="6" t="n"/>
+      <c r="B485" s="5" t="n"/>
+      <c r="C485" s="7" t="n"/>
+      <c r="D485" s="7" t="n"/>
+      <c r="E485" s="5" t="n"/>
+    </row>
+    <row r="486">
+      <c r="A486" s="6" t="n"/>
+      <c r="B486" s="5" t="n"/>
+      <c r="C486" s="7" t="n"/>
+      <c r="D486" s="7" t="n"/>
+      <c r="E486" s="5" t="n"/>
+    </row>
+    <row r="487">
+      <c r="A487" s="6" t="n"/>
+      <c r="B487" s="5" t="n"/>
+      <c r="C487" s="7" t="n"/>
+      <c r="D487" s="7" t="n"/>
+      <c r="E487" s="5" t="n"/>
+    </row>
+    <row r="488">
+      <c r="A488" s="6" t="n"/>
+      <c r="B488" s="5" t="n"/>
+      <c r="C488" s="7" t="n"/>
+      <c r="D488" s="7" t="n"/>
+      <c r="E488" s="5" t="n"/>
+    </row>
+    <row r="489">
+      <c r="A489" s="6" t="n"/>
+      <c r="B489" s="5" t="n"/>
+      <c r="C489" s="7" t="n"/>
+      <c r="D489" s="7" t="n"/>
+      <c r="E489" s="5" t="n"/>
+    </row>
+    <row r="490">
+      <c r="A490" s="6" t="n"/>
+      <c r="B490" s="5" t="n"/>
+      <c r="C490" s="7" t="n"/>
+      <c r="D490" s="7" t="n"/>
+      <c r="E490" s="5" t="n"/>
+    </row>
+    <row r="491">
+      <c r="A491" s="6" t="n"/>
+      <c r="B491" s="5" t="n"/>
+      <c r="C491" s="7" t="n"/>
+      <c r="D491" s="7" t="n"/>
+      <c r="E491" s="5" t="n"/>
+    </row>
+    <row r="492">
+      <c r="A492" s="6" t="n"/>
+      <c r="B492" s="5" t="n"/>
+      <c r="C492" s="7" t="n"/>
+      <c r="D492" s="7" t="n"/>
+      <c r="E492" s="5" t="n"/>
+    </row>
+    <row r="493">
+      <c r="A493" s="6" t="n"/>
+      <c r="B493" s="5" t="n"/>
+      <c r="C493" s="7" t="n"/>
+      <c r="D493" s="7" t="n"/>
+      <c r="E493" s="5" t="n"/>
+    </row>
+    <row r="494">
+      <c r="A494" s="6" t="n"/>
+      <c r="B494" s="5" t="n"/>
+      <c r="C494" s="7" t="n"/>
+      <c r="D494" s="7" t="n"/>
+      <c r="E494" s="5" t="n"/>
+    </row>
+    <row r="495">
+      <c r="A495" s="6" t="n"/>
+      <c r="B495" s="5" t="n"/>
+      <c r="C495" s="7" t="n"/>
+      <c r="D495" s="7" t="n"/>
+      <c r="E495" s="5" t="n"/>
+    </row>
+    <row r="496">
+      <c r="A496" s="6" t="n"/>
+      <c r="B496" s="5" t="n"/>
+      <c r="C496" s="7" t="n"/>
+      <c r="D496" s="7" t="n"/>
+      <c r="E496" s="5" t="n"/>
+    </row>
+    <row r="497">
+      <c r="A497" s="6" t="n"/>
+      <c r="B497" s="5" t="n"/>
+      <c r="C497" s="7" t="n"/>
+      <c r="D497" s="7" t="n"/>
+      <c r="E497" s="5" t="n"/>
+    </row>
+    <row r="498">
+      <c r="A498" s="6" t="n"/>
+      <c r="B498" s="5" t="n"/>
+      <c r="C498" s="7" t="n"/>
+      <c r="D498" s="7" t="n"/>
+      <c r="E498" s="5" t="n"/>
+    </row>
+    <row r="499">
+      <c r="A499" s="6" t="n"/>
+      <c r="B499" s="5" t="n"/>
+      <c r="C499" s="7" t="n"/>
+      <c r="D499" s="7" t="n"/>
+      <c r="E499" s="5" t="n"/>
+    </row>
+    <row r="500">
+      <c r="A500" s="6" t="n"/>
+      <c r="B500" s="5" t="n"/>
+      <c r="C500" s="7" t="n"/>
+      <c r="D500" s="7" t="n"/>
+      <c r="E500" s="5" t="n"/>
+    </row>
+    <row r="501">
+      <c r="A501" s="6" t="n"/>
+      <c r="B501" s="5" t="n"/>
+      <c r="C501" s="7" t="n"/>
+      <c r="D501" s="7" t="n"/>
+      <c r="E501" s="5" t="n"/>
+    </row>
+    <row r="502">
+      <c r="A502" s="6" t="n"/>
+      <c r="B502" s="5" t="n"/>
+      <c r="C502" s="7" t="n"/>
+      <c r="D502" s="7" t="n"/>
+      <c r="E502" s="5" t="n"/>
+    </row>
+    <row r="503">
+      <c r="A503" s="6" t="n"/>
+      <c r="B503" s="5" t="n"/>
+      <c r="C503" s="7" t="n"/>
+      <c r="D503" s="7" t="n"/>
+      <c r="E503" s="5" t="n"/>
+    </row>
+    <row r="504">
+      <c r="A504" s="6" t="n"/>
+      <c r="B504" s="5" t="n"/>
+      <c r="C504" s="7" t="n"/>
+      <c r="D504" s="7" t="n"/>
+      <c r="E504" s="5" t="n"/>
+    </row>
+    <row r="505">
+      <c r="A505" s="6" t="n"/>
+      <c r="B505" s="5" t="n"/>
+      <c r="C505" s="7" t="n"/>
+      <c r="D505" s="7" t="n"/>
+      <c r="E505" s="5" t="n"/>
+    </row>
+    <row r="506">
+      <c r="A506" s="6" t="n"/>
+      <c r="B506" s="5" t="n"/>
+      <c r="C506" s="7" t="n"/>
+      <c r="D506" s="7" t="n"/>
+      <c r="E506" s="5" t="n"/>
+    </row>
+    <row r="507">
+      <c r="A507" s="6" t="n"/>
+      <c r="B507" s="5" t="n"/>
+      <c r="C507" s="7" t="n"/>
+      <c r="D507" s="7" t="n"/>
+      <c r="E507" s="5" t="n"/>
+    </row>
+    <row r="508">
+      <c r="A508" s="6" t="n"/>
+      <c r="B508" s="5" t="n"/>
+      <c r="C508" s="7" t="n"/>
+      <c r="D508" s="7" t="n"/>
+      <c r="E508" s="5" t="n"/>
+    </row>
+    <row r="509">
+      <c r="A509" s="6" t="n"/>
+      <c r="B509" s="5" t="n"/>
+      <c r="C509" s="7" t="n"/>
+      <c r="D509" s="7" t="n"/>
+      <c r="E509" s="5" t="n"/>
+    </row>
+    <row r="510">
+      <c r="A510" s="6" t="n"/>
+      <c r="B510" s="5" t="n"/>
+      <c r="C510" s="7" t="n"/>
+      <c r="D510" s="7" t="n"/>
+      <c r="E510" s="5" t="n"/>
+    </row>
+    <row r="511">
+      <c r="A511" s="6" t="n"/>
+      <c r="B511" s="5" t="n"/>
+      <c r="C511" s="7" t="n"/>
+      <c r="D511" s="7" t="n"/>
+      <c r="E511" s="5" t="n"/>
+    </row>
+    <row r="512">
+      <c r="A512" s="6" t="n"/>
+      <c r="B512" s="5" t="n"/>
+      <c r="C512" s="7" t="n"/>
+      <c r="D512" s="7" t="n"/>
+      <c r="E512" s="5" t="n"/>
+    </row>
+    <row r="513">
+      <c r="A513" s="6" t="n"/>
+      <c r="B513" s="5" t="n"/>
+      <c r="C513" s="7" t="n"/>
+      <c r="D513" s="7" t="n"/>
+      <c r="E513" s="5" t="n"/>
+    </row>
+    <row r="514">
+      <c r="A514" s="6" t="n"/>
+      <c r="B514" s="5" t="n"/>
+      <c r="C514" s="7" t="n"/>
+      <c r="D514" s="7" t="n"/>
+      <c r="E514" s="5" t="n"/>
+    </row>
+    <row r="515">
+      <c r="A515" s="6" t="n"/>
+      <c r="B515" s="5" t="n"/>
+      <c r="C515" s="7" t="n"/>
+      <c r="D515" s="7" t="n"/>
+      <c r="E515" s="5" t="n"/>
+    </row>
+    <row r="516">
+      <c r="A516" s="6" t="n"/>
+      <c r="B516" s="5" t="n"/>
+      <c r="C516" s="7" t="n"/>
+      <c r="D516" s="7" t="n"/>
+      <c r="E516" s="5" t="n"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="6" t="n"/>
+      <c r="B517" s="5" t="n"/>
+      <c r="C517" s="7" t="n"/>
+      <c r="D517" s="7" t="n"/>
+      <c r="E517" s="5" t="n"/>
+    </row>
+    <row r="518">
+      <c r="A518" s="6" t="n"/>
+      <c r="B518" s="5" t="n"/>
+      <c r="C518" s="7" t="n"/>
+      <c r="D518" s="7" t="n"/>
+      <c r="E518" s="5" t="n"/>
+    </row>
+    <row r="519">
+      <c r="A519" s="6" t="n"/>
+      <c r="B519" s="5" t="n"/>
+      <c r="C519" s="7" t="n"/>
+      <c r="D519" s="7" t="n"/>
+      <c r="E519" s="5" t="n"/>
+    </row>
+    <row r="520">
+      <c r="A520" s="6" t="n"/>
+      <c r="B520" s="5" t="n"/>
+      <c r="C520" s="7" t="n"/>
+      <c r="D520" s="7" t="n"/>
+      <c r="E520" s="5" t="n"/>
+    </row>
+    <row r="521">
+      <c r="A521" s="6" t="n"/>
+      <c r="B521" s="5" t="n"/>
+      <c r="C521" s="7" t="n"/>
+      <c r="D521" s="7" t="n"/>
+      <c r="E521" s="5" t="n"/>
+    </row>
+    <row r="522">
+      <c r="A522" s="6" t="n"/>
+      <c r="B522" s="5" t="n"/>
+      <c r="C522" s="7" t="n"/>
+      <c r="D522" s="7" t="n"/>
+      <c r="E522" s="5" t="n"/>
+    </row>
+    <row r="523">
+      <c r="A523" s="6" t="n"/>
+      <c r="B523" s="5" t="n"/>
+      <c r="C523" s="7" t="n"/>
+      <c r="D523" s="7" t="n"/>
+      <c r="E523" s="5" t="n"/>
+    </row>
+    <row r="524">
+      <c r="A524" s="6" t="n"/>
+      <c r="B524" s="5" t="n"/>
+      <c r="C524" s="7" t="n"/>
+      <c r="D524" s="7" t="n"/>
+      <c r="E524" s="5" t="n"/>
+    </row>
+    <row r="525">
+      <c r="A525" s="6" t="n"/>
+      <c r="B525" s="5" t="n"/>
+      <c r="C525" s="7" t="n"/>
+      <c r="D525" s="7" t="n"/>
+      <c r="E525" s="5" t="n"/>
+    </row>
+    <row r="526">
+      <c r="A526" s="6" t="n"/>
+      <c r="B526" s="5" t="n"/>
+      <c r="C526" s="7" t="n"/>
+      <c r="D526" s="7" t="n"/>
+      <c r="E526" s="5" t="n"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="6" t="n"/>
+      <c r="B527" s="5" t="n"/>
+      <c r="C527" s="7" t="n"/>
+      <c r="D527" s="7" t="n"/>
+      <c r="E527" s="5" t="n"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="6" t="n"/>
+      <c r="B528" s="5" t="n"/>
+      <c r="C528" s="7" t="n"/>
+      <c r="D528" s="7" t="n"/>
+      <c r="E528" s="5" t="n"/>
+    </row>
+    <row r="529">
+      <c r="A529" s="6" t="n"/>
+      <c r="B529" s="5" t="n"/>
+      <c r="C529" s="7" t="n"/>
+      <c r="D529" s="7" t="n"/>
+      <c r="E529" s="5" t="n"/>
+    </row>
+    <row r="530">
+      <c r="A530" s="6" t="n"/>
+      <c r="B530" s="5" t="n"/>
+      <c r="C530" s="7" t="n"/>
+      <c r="D530" s="7" t="n"/>
+      <c r="E530" s="5" t="n"/>
+    </row>
+    <row r="531">
+      <c r="A531" s="6" t="n"/>
+      <c r="B531" s="5" t="n"/>
+      <c r="C531" s="7" t="n"/>
+      <c r="D531" s="7" t="n"/>
+      <c r="E531" s="5" t="n"/>
+    </row>
+    <row r="532">
+      <c r="A532" s="6" t="n"/>
+      <c r="B532" s="5" t="n"/>
+      <c r="C532" s="7" t="n"/>
+      <c r="D532" s="7" t="n"/>
+      <c r="E532" s="5" t="n"/>
+    </row>
+    <row r="533">
+      <c r="A533" s="6" t="n"/>
+      <c r="B533" s="5" t="n"/>
+      <c r="C533" s="7" t="n"/>
+      <c r="D533" s="7" t="n"/>
+      <c r="E533" s="5" t="n"/>
+    </row>
+    <row r="534">
+      <c r="A534" s="6" t="n"/>
+      <c r="B534" s="5" t="n"/>
+      <c r="C534" s="7" t="n"/>
+      <c r="D534" s="7" t="n"/>
+      <c r="E534" s="5" t="n"/>
+    </row>
+    <row r="535">
+      <c r="A535" s="6" t="n"/>
+      <c r="B535" s="5" t="n"/>
+      <c r="C535" s="7" t="n"/>
+      <c r="D535" s="7" t="n"/>
+      <c r="E535" s="5" t="n"/>
+    </row>
+    <row r="536">
+      <c r="A536" s="6" t="n"/>
+      <c r="B536" s="5" t="n"/>
+      <c r="C536" s="7" t="n"/>
+      <c r="D536" s="7" t="n"/>
+      <c r="E536" s="5" t="n"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="6" t="n"/>
+      <c r="B537" s="5" t="n"/>
+      <c r="C537" s="7" t="n"/>
+      <c r="D537" s="7" t="n"/>
+      <c r="E537" s="5" t="n"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="6" t="n"/>
+      <c r="B538" s="5" t="n"/>
+      <c r="C538" s="7" t="n"/>
+      <c r="D538" s="7" t="n"/>
+      <c r="E538" s="5" t="n"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="6" t="n"/>
+      <c r="B539" s="5" t="n"/>
+      <c r="C539" s="7" t="n"/>
+      <c r="D539" s="7" t="n"/>
+      <c r="E539" s="5" t="n"/>
+    </row>
+    <row r="540">
+      <c r="A540" s="6" t="n"/>
+      <c r="B540" s="5" t="n"/>
+      <c r="C540" s="7" t="n"/>
+      <c r="D540" s="7" t="n"/>
+      <c r="E540" s="5" t="n"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="6" t="n"/>
+      <c r="B541" s="5" t="n"/>
+      <c r="C541" s="7" t="n"/>
+      <c r="D541" s="7" t="n"/>
+      <c r="E541" s="5" t="n"/>
+    </row>
+    <row r="542">
+      <c r="A542" s="6" t="n"/>
+      <c r="B542" s="5" t="n"/>
+      <c r="C542" s="7" t="n"/>
+      <c r="D542" s="7" t="n"/>
+      <c r="E542" s="5" t="n"/>
+    </row>
+    <row r="543">
+      <c r="A543" s="6" t="n"/>
+      <c r="B543" s="5" t="n"/>
+      <c r="C543" s="7" t="n"/>
+      <c r="D543" s="7" t="n"/>
+      <c r="E543" s="5" t="n"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="6" t="n"/>
+      <c r="B544" s="5" t="n"/>
+      <c r="C544" s="7" t="n"/>
+      <c r="D544" s="7" t="n"/>
+      <c r="E544" s="5" t="n"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="6" t="n"/>
+      <c r="B545" s="5" t="n"/>
+      <c r="C545" s="7" t="n"/>
+      <c r="D545" s="7" t="n"/>
+      <c r="E545" s="5" t="n"/>
+    </row>
+    <row r="546">
+      <c r="A546" s="6" t="n"/>
+      <c r="B546" s="5" t="n"/>
+      <c r="C546" s="7" t="n"/>
+      <c r="D546" s="7" t="n"/>
+      <c r="E546" s="5" t="n"/>
+    </row>
+    <row r="547">
+      <c r="A547" s="6" t="n"/>
+      <c r="B547" s="5" t="n"/>
+      <c r="C547" s="7" t="n"/>
+      <c r="D547" s="7" t="n"/>
+      <c r="E547" s="5" t="n"/>
+    </row>
+    <row r="548">
+      <c r="A548" s="6" t="n"/>
+      <c r="B548" s="5" t="n"/>
+      <c r="C548" s="7" t="n"/>
+      <c r="D548" s="7" t="n"/>
+      <c r="E548" s="5" t="n"/>
+    </row>
+    <row r="549">
+      <c r="A549" s="6" t="n"/>
+      <c r="B549" s="5" t="n"/>
+      <c r="C549" s="7" t="n"/>
+      <c r="D549" s="7" t="n"/>
+      <c r="E549" s="5" t="n"/>
+    </row>
+    <row r="550">
+      <c r="A550" s="6" t="n"/>
+      <c r="B550" s="5" t="n"/>
+      <c r="C550" s="7" t="n"/>
+      <c r="D550" s="7" t="n"/>
+      <c r="E550" s="5" t="n"/>
+    </row>
+    <row r="551">
+      <c r="A551" s="6" t="n"/>
+      <c r="B551" s="5" t="n"/>
+      <c r="C551" s="7" t="n"/>
+      <c r="D551" s="7" t="n"/>
+      <c r="E551" s="5" t="n"/>
+    </row>
+    <row r="552">
+      <c r="A552" s="6" t="n"/>
+      <c r="B552" s="5" t="n"/>
+      <c r="C552" s="7" t="n"/>
+      <c r="D552" s="7" t="n"/>
+      <c r="E552" s="5" t="n"/>
+    </row>
+    <row r="553">
+      <c r="A553" s="6" t="n"/>
+      <c r="B553" s="5" t="n"/>
+      <c r="C553" s="7" t="n"/>
+      <c r="D553" s="7" t="n"/>
+      <c r="E553" s="5" t="n"/>
+    </row>
+    <row r="554">
+      <c r="A554" s="6" t="n"/>
+      <c r="B554" s="5" t="n"/>
+      <c r="C554" s="7" t="n"/>
+      <c r="D554" s="7" t="n"/>
+      <c r="E554" s="5" t="n"/>
+    </row>
+    <row r="555">
+      <c r="A555" s="6" t="n"/>
+      <c r="B555" s="5" t="n"/>
+      <c r="C555" s="7" t="n"/>
+      <c r="D555" s="7" t="n"/>
+      <c r="E555" s="5" t="n"/>
+    </row>
+    <row r="556">
+      <c r="A556" s="6" t="n"/>
+      <c r="B556" s="5" t="n"/>
+      <c r="C556" s="7" t="n"/>
+      <c r="D556" s="7" t="n"/>
+      <c r="E556" s="5" t="n"/>
+    </row>
+    <row r="557">
+      <c r="A557" s="6" t="n"/>
+      <c r="B557" s="5" t="n"/>
+      <c r="C557" s="7" t="n"/>
+      <c r="D557" s="7" t="n"/>
+      <c r="E557" s="5" t="n"/>
+    </row>
+    <row r="558">
+      <c r="A558" s="6" t="n"/>
+      <c r="B558" s="5" t="n"/>
+      <c r="C558" s="7" t="n"/>
+      <c r="D558" s="7" t="n"/>
+      <c r="E558" s="5" t="n"/>
+    </row>
+    <row r="559">
+      <c r="A559" s="6" t="n"/>
+      <c r="B559" s="5" t="n"/>
+      <c r="C559" s="7" t="n"/>
+      <c r="D559" s="7" t="n"/>
+      <c r="E559" s="5" t="n"/>
+    </row>
+    <row r="560">
+      <c r="A560" s="6" t="n"/>
+      <c r="B560" s="5" t="n"/>
+      <c r="C560" s="7" t="n"/>
+      <c r="D560" s="7" t="n"/>
+      <c r="E560" s="5" t="n"/>
+    </row>
+    <row r="561">
+      <c r="A561" s="6" t="n"/>
+      <c r="B561" s="5" t="n"/>
+      <c r="C561" s="7" t="n"/>
+      <c r="D561" s="7" t="n"/>
+      <c r="E561" s="5" t="n"/>
+    </row>
+    <row r="562">
+      <c r="A562" s="6" t="n"/>
+      <c r="B562" s="5" t="n"/>
+      <c r="C562" s="7" t="n"/>
+      <c r="D562" s="7" t="n"/>
+      <c r="E562" s="5" t="n"/>
+    </row>
+    <row r="563">
+      <c r="A563" s="6" t="n"/>
+      <c r="B563" s="5" t="n"/>
+      <c r="C563" s="7" t="n"/>
+      <c r="D563" s="7" t="n"/>
+      <c r="E563" s="5" t="n"/>
+    </row>
+    <row r="564">
+      <c r="A564" s="6" t="n"/>
+      <c r="B564" s="5" t="n"/>
+      <c r="C564" s="7" t="n"/>
+      <c r="D564" s="7" t="n"/>
+      <c r="E564" s="5" t="n"/>
+    </row>
+    <row r="565">
+      <c r="A565" s="6" t="n"/>
+      <c r="B565" s="5" t="n"/>
+      <c r="C565" s="7" t="n"/>
+      <c r="D565" s="7" t="n"/>
+      <c r="E565" s="5" t="n"/>
+    </row>
+    <row r="566">
+      <c r="A566" s="6" t="n"/>
+      <c r="B566" s="5" t="n"/>
+      <c r="C566" s="7" t="n"/>
+      <c r="D566" s="7" t="n"/>
+      <c r="E566" s="5" t="n"/>
+    </row>
+    <row r="567">
+      <c r="A567" s="6" t="n"/>
+      <c r="B567" s="5" t="n"/>
+      <c r="C567" s="7" t="n"/>
+      <c r="D567" s="7" t="n"/>
+      <c r="E567" s="5" t="n"/>
+    </row>
+    <row r="568">
+      <c r="A568" s="6" t="n"/>
+      <c r="B568" s="5" t="n"/>
+      <c r="C568" s="7" t="n"/>
+      <c r="D568" s="7" t="n"/>
+      <c r="E568" s="5" t="n"/>
+    </row>
+    <row r="569">
+      <c r="A569" s="6" t="n"/>
+      <c r="B569" s="5" t="n"/>
+      <c r="C569" s="7" t="n"/>
+      <c r="D569" s="7" t="n"/>
+      <c r="E569" s="5" t="n"/>
+    </row>
+    <row r="570">
+      <c r="A570" s="6" t="n"/>
+      <c r="B570" s="5" t="n"/>
+      <c r="C570" s="7" t="n"/>
+      <c r="D570" s="7" t="n"/>
+      <c r="E570" s="5" t="n"/>
+    </row>
+    <row r="571">
+      <c r="A571" s="6" t="n"/>
+      <c r="B571" s="5" t="n"/>
+      <c r="C571" s="7" t="n"/>
+      <c r="D571" s="7" t="n"/>
+      <c r="E571" s="5" t="n"/>
+    </row>
+    <row r="572">
+      <c r="A572" s="6" t="n"/>
+      <c r="B572" s="5" t="n"/>
+      <c r="C572" s="7" t="n"/>
+      <c r="D572" s="7" t="n"/>
+      <c r="E572" s="5" t="n"/>
+    </row>
+    <row r="573">
+      <c r="A573" s="6" t="n"/>
+      <c r="B573" s="5" t="n"/>
+      <c r="C573" s="7" t="n"/>
+      <c r="D573" s="7" t="n"/>
+      <c r="E573" s="5" t="n"/>
+    </row>
+    <row r="574">
+      <c r="A574" s="6" t="n"/>
+      <c r="B574" s="5" t="n"/>
+      <c r="C574" s="7" t="n"/>
+      <c r="D574" s="7" t="n"/>
+      <c r="E574" s="5" t="n"/>
+    </row>
+    <row r="575">
+      <c r="A575" s="6" t="n"/>
+      <c r="B575" s="5" t="n"/>
+      <c r="C575" s="7" t="n"/>
+      <c r="D575" s="7" t="n"/>
+      <c r="E575" s="5" t="n"/>
+    </row>
+    <row r="576">
+      <c r="A576" s="6" t="n"/>
+      <c r="B576" s="5" t="n"/>
+      <c r="C576" s="7" t="n"/>
+      <c r="D576" s="7" t="n"/>
+      <c r="E576" s="5" t="n"/>
+    </row>
+    <row r="577">
+      <c r="A577" s="6" t="n"/>
+      <c r="B577" s="5" t="n"/>
+      <c r="C577" s="7" t="n"/>
+      <c r="D577" s="7" t="n"/>
+      <c r="E577" s="5" t="n"/>
+    </row>
+    <row r="578">
+      <c r="A578" s="6" t="n"/>
+      <c r="B578" s="5" t="n"/>
+      <c r="C578" s="7" t="n"/>
+      <c r="D578" s="7" t="n"/>
+      <c r="E578" s="5" t="n"/>
+    </row>
+    <row r="579">
+      <c r="A579" s="6" t="n"/>
+      <c r="B579" s="5" t="n"/>
+      <c r="C579" s="7" t="n"/>
+      <c r="D579" s="7" t="n"/>
+      <c r="E579" s="5" t="n"/>
+    </row>
+    <row r="580">
+      <c r="A580" s="6" t="n"/>
+      <c r="B580" s="5" t="n"/>
+      <c r="C580" s="7" t="n"/>
+      <c r="D580" s="7" t="n"/>
+      <c r="E580" s="5" t="n"/>
+    </row>
+    <row r="581">
+      <c r="A581" s="6" t="n"/>
+      <c r="B581" s="5" t="n"/>
+      <c r="C581" s="7" t="n"/>
+      <c r="D581" s="7" t="n"/>
+      <c r="E581" s="5" t="n"/>
+    </row>
+    <row r="582">
+      <c r="A582" s="6" t="n"/>
+      <c r="B582" s="5" t="n"/>
+      <c r="C582" s="7" t="n"/>
+      <c r="D582" s="7" t="n"/>
+      <c r="E582" s="5" t="n"/>
+    </row>
+    <row r="583">
+      <c r="A583" s="6" t="n"/>
+      <c r="B583" s="5" t="n"/>
+      <c r="C583" s="7" t="n"/>
+      <c r="D583" s="7" t="n"/>
+      <c r="E583" s="5" t="n"/>
+    </row>
+    <row r="584">
+      <c r="A584" s="6" t="n"/>
+      <c r="B584" s="5" t="n"/>
+      <c r="C584" s="7" t="n"/>
+      <c r="D584" s="7" t="n"/>
+      <c r="E584" s="5" t="n"/>
+    </row>
+    <row r="585">
+      <c r="A585" s="6" t="n"/>
+      <c r="B585" s="5" t="n"/>
+      <c r="C585" s="7" t="n"/>
+      <c r="D585" s="7" t="n"/>
+      <c r="E585" s="5" t="n"/>
+    </row>
+    <row r="586">
+      <c r="A586" s="6" t="n"/>
+      <c r="B586" s="5" t="n"/>
+      <c r="C586" s="7" t="n"/>
+      <c r="D586" s="7" t="n"/>
+      <c r="E586" s="5" t="n"/>
+    </row>
+    <row r="587">
+      <c r="A587" s="6" t="n"/>
+      <c r="B587" s="5" t="n"/>
+      <c r="C587" s="7" t="n"/>
+      <c r="D587" s="7" t="n"/>
+      <c r="E587" s="5" t="n"/>
+    </row>
+    <row r="588">
+      <c r="A588" s="6" t="n"/>
+      <c r="B588" s="5" t="n"/>
+      <c r="C588" s="7" t="n"/>
+      <c r="D588" s="7" t="n"/>
+      <c r="E588" s="5" t="n"/>
+    </row>
+    <row r="589">
+      <c r="A589" s="6" t="n"/>
+      <c r="B589" s="5" t="n"/>
+      <c r="C589" s="7" t="n"/>
+      <c r="D589" s="7" t="n"/>
+      <c r="E589" s="5" t="n"/>
+    </row>
+    <row r="590">
+      <c r="A590" s="6" t="n"/>
+      <c r="B590" s="5" t="n"/>
+      <c r="C590" s="7" t="n"/>
+      <c r="D590" s="7" t="n"/>
+      <c r="E590" s="5" t="n"/>
+    </row>
+    <row r="591">
+      <c r="A591" s="6" t="n"/>
+      <c r="B591" s="5" t="n"/>
+      <c r="C591" s="7" t="n"/>
+      <c r="D591" s="7" t="n"/>
+      <c r="E591" s="5" t="n"/>
+    </row>
+    <row r="592">
+      <c r="A592" s="6" t="n"/>
+      <c r="B592" s="5" t="n"/>
+      <c r="C592" s="7" t="n"/>
+      <c r="D592" s="7" t="n"/>
+      <c r="E592" s="5" t="n"/>
+    </row>
+    <row r="593">
+      <c r="A593" s="6" t="n"/>
+      <c r="B593" s="5" t="n"/>
+      <c r="C593" s="7" t="n"/>
+      <c r="D593" s="7" t="n"/>
+      <c r="E593" s="5" t="n"/>
+    </row>
+    <row r="594">
+      <c r="A594" s="6" t="n"/>
+      <c r="B594" s="5" t="n"/>
+      <c r="C594" s="7" t="n"/>
+      <c r="D594" s="7" t="n"/>
+      <c r="E594" s="5" t="n"/>
+    </row>
+    <row r="595">
+      <c r="A595" s="6" t="n"/>
+      <c r="B595" s="5" t="n"/>
+      <c r="C595" s="7" t="n"/>
+      <c r="D595" s="7" t="n"/>
+      <c r="E595" s="5" t="n"/>
+    </row>
+    <row r="596">
+      <c r="A596" s="6" t="n"/>
+      <c r="B596" s="5" t="n"/>
+      <c r="C596" s="7" t="n"/>
+      <c r="D596" s="7" t="n"/>
+      <c r="E596" s="5" t="n"/>
+    </row>
+    <row r="597">
+      <c r="A597" s="6" t="n"/>
+      <c r="B597" s="5" t="n"/>
+      <c r="C597" s="7" t="n"/>
+      <c r="D597" s="7" t="n"/>
+      <c r="E597" s="5" t="n"/>
+    </row>
+    <row r="598">
+      <c r="A598" s="6" t="n"/>
+      <c r="B598" s="5" t="n"/>
+      <c r="C598" s="7" t="n"/>
+      <c r="D598" s="7" t="n"/>
+      <c r="E598" s="5" t="n"/>
+    </row>
+    <row r="599">
+      <c r="A599" s="6" t="n"/>
+      <c r="B599" s="5" t="n"/>
+      <c r="C599" s="7" t="n"/>
+      <c r="D599" s="7" t="n"/>
+      <c r="E599" s="5" t="n"/>
+    </row>
+    <row r="600">
+      <c r="A600" s="6" t="n"/>
+      <c r="B600" s="5" t="n"/>
+      <c r="C600" s="7" t="n"/>
+      <c r="D600" s="7" t="n"/>
+      <c r="E600" s="5" t="n"/>
+    </row>
+    <row r="601">
+      <c r="A601" s="6" t="n"/>
+      <c r="B601" s="5" t="n"/>
+      <c r="C601" s="7" t="n"/>
+      <c r="D601" s="7" t="n"/>
+      <c r="E601" s="5" t="n"/>
+    </row>
+    <row r="602">
+      <c r="A602" s="6" t="n"/>
+      <c r="B602" s="5" t="n"/>
+      <c r="C602" s="7" t="n"/>
+      <c r="D602" s="7" t="n"/>
+      <c r="E602" s="5" t="n"/>
+    </row>
+    <row r="603">
+      <c r="A603" s="6" t="n"/>
+      <c r="B603" s="5" t="n"/>
+      <c r="C603" s="7" t="n"/>
+      <c r="D603" s="7" t="n"/>
+      <c r="E603" s="5" t="n"/>
+    </row>
+    <row r="604">
+      <c r="A604" s="6" t="n"/>
+      <c r="B604" s="5" t="n"/>
+      <c r="C604" s="7" t="n"/>
+      <c r="D604" s="7" t="n"/>
+      <c r="E604" s="5" t="n"/>
+    </row>
+    <row r="605">
+      <c r="A605" s="6" t="n"/>
+      <c r="B605" s="5" t="n"/>
+      <c r="C605" s="7" t="n"/>
+      <c r="D605" s="7" t="n"/>
+      <c r="E605" s="5" t="n"/>
+    </row>
+    <row r="606">
+      <c r="A606" s="6" t="n"/>
+      <c r="B606" s="5" t="n"/>
+      <c r="C606" s="7" t="n"/>
+      <c r="D606" s="7" t="n"/>
+      <c r="E606" s="5" t="n"/>
+    </row>
+    <row r="607">
+      <c r="A607" s="6" t="n"/>
+      <c r="B607" s="5" t="n"/>
+      <c r="C607" s="7" t="n"/>
+      <c r="D607" s="7" t="n"/>
+      <c r="E607" s="5" t="n"/>
+    </row>
+    <row r="608">
+      <c r="A608" s="6" t="n"/>
+      <c r="B608" s="5" t="n"/>
+      <c r="C608" s="7" t="n"/>
+      <c r="D608" s="7" t="n"/>
+      <c r="E608" s="5" t="n"/>
+    </row>
+    <row r="609">
+      <c r="A609" s="6" t="n"/>
+      <c r="B609" s="5" t="n"/>
+      <c r="C609" s="7" t="n"/>
+      <c r="D609" s="7" t="n"/>
+      <c r="E609" s="5" t="n"/>
+    </row>
+    <row r="610">
+      <c r="A610" s="6" t="n"/>
+      <c r="B610" s="5" t="n"/>
+      <c r="C610" s="7" t="n"/>
+      <c r="D610" s="7" t="n"/>
+      <c r="E610" s="5" t="n"/>
+    </row>
+    <row r="611">
+      <c r="A611" s="6" t="n"/>
+      <c r="B611" s="5" t="n"/>
+      <c r="C611" s="7" t="n"/>
+      <c r="D611" s="7" t="n"/>
+      <c r="E611" s="5" t="n"/>
+    </row>
+    <row r="612">
+      <c r="A612" s="6" t="n"/>
+      <c r="B612" s="5" t="n"/>
+      <c r="C612" s="7" t="n"/>
+      <c r="D612" s="7" t="n"/>
+      <c r="E612" s="5" t="n"/>
+    </row>
+    <row r="613">
+      <c r="A613" s="6" t="n"/>
+      <c r="B613" s="5" t="n"/>
+      <c r="C613" s="7" t="n"/>
+      <c r="D613" s="7" t="n"/>
+      <c r="E613" s="5" t="n"/>
+    </row>
+    <row r="614">
+      <c r="A614" s="6" t="n"/>
+      <c r="B614" s="5" t="n"/>
+      <c r="C614" s="7" t="n"/>
+      <c r="D614" s="7" t="n"/>
+      <c r="E614" s="5" t="n"/>
+    </row>
+    <row r="615">
+      <c r="A615" s="6" t="n"/>
+      <c r="B615" s="5" t="n"/>
+      <c r="C615" s="7" t="n"/>
+      <c r="D615" s="7" t="n"/>
+      <c r="E615" s="5" t="n"/>
+    </row>
+    <row r="616">
+      <c r="A616" s="6" t="n"/>
+      <c r="B616" s="5" t="n"/>
+      <c r="C616" s="7" t="n"/>
+      <c r="D616" s="7" t="n"/>
+      <c r="E616" s="5" t="n"/>
+    </row>
+    <row r="617">
+      <c r="A617" s="6" t="n"/>
+      <c r="B617" s="5" t="n"/>
+      <c r="C617" s="7" t="n"/>
+      <c r="D617" s="7" t="n"/>
+      <c r="E617" s="5" t="n"/>
+    </row>
+    <row r="618">
+      <c r="A618" s="6" t="n"/>
+      <c r="B618" s="5" t="n"/>
+      <c r="C618" s="7" t="n"/>
+      <c r="D618" s="7" t="n"/>
+      <c r="E618" s="5" t="n"/>
+    </row>
+    <row r="619">
+      <c r="A619" s="6" t="n"/>
+      <c r="B619" s="5" t="n"/>
+      <c r="C619" s="7" t="n"/>
+      <c r="D619" s="7" t="n"/>
+      <c r="E619" s="5" t="n"/>
+    </row>
+    <row r="620">
+      <c r="A620" s="6" t="n"/>
+      <c r="B620" s="5" t="n"/>
+      <c r="C620" s="7" t="n"/>
+      <c r="D620" s="7" t="n"/>
+      <c r="E620" s="5" t="n"/>
+    </row>
+    <row r="621">
+      <c r="A621" s="6" t="n"/>
+      <c r="B621" s="5" t="n"/>
+      <c r="C621" s="7" t="n"/>
+      <c r="D621" s="7" t="n"/>
+      <c r="E621" s="5" t="n"/>
+    </row>
+    <row r="622">
+      <c r="A622" s="6" t="n"/>
+      <c r="B622" s="5" t="n"/>
+      <c r="C622" s="7" t="n"/>
+      <c r="D622" s="7" t="n"/>
+      <c r="E622" s="5" t="n"/>
+    </row>
+    <row r="623">
+      <c r="A623" s="6" t="n"/>
+      <c r="B623" s="5" t="n"/>
+      <c r="C623" s="7" t="n"/>
+      <c r="D623" s="7" t="n"/>
+      <c r="E623" s="5" t="n"/>
+    </row>
+    <row r="624">
+      <c r="A624" s="6" t="n"/>
+      <c r="B624" s="5" t="n"/>
+      <c r="C624" s="7" t="n"/>
+      <c r="D624" s="7" t="n"/>
+      <c r="E624" s="5" t="n"/>
+    </row>
+    <row r="625">
+      <c r="A625" s="6" t="n"/>
+      <c r="B625" s="5" t="n"/>
+      <c r="C625" s="7" t="n"/>
+      <c r="D625" s="7" t="n"/>
+      <c r="E625" s="5" t="n"/>
+    </row>
+    <row r="626">
+      <c r="A626" s="6" t="n"/>
+      <c r="B626" s="5" t="n"/>
+      <c r="C626" s="7" t="n"/>
+      <c r="D626" s="7" t="n"/>
+      <c r="E626" s="5" t="n"/>
+    </row>
+    <row r="627">
+      <c r="A627" s="6" t="n"/>
+      <c r="B627" s="5" t="n"/>
+      <c r="C627" s="7" t="n"/>
+      <c r="D627" s="7" t="n"/>
+      <c r="E627" s="5" t="n"/>
+    </row>
+    <row r="628">
+      <c r="A628" s="6" t="n"/>
+      <c r="B628" s="5" t="n"/>
+      <c r="C628" s="7" t="n"/>
+      <c r="D628" s="7" t="n"/>
+      <c r="E628" s="5" t="n"/>
+    </row>
+    <row r="629">
+      <c r="A629" s="6" t="n"/>
+      <c r="B629" s="5" t="n"/>
+      <c r="C629" s="7" t="n"/>
+      <c r="D629" s="7" t="n"/>
+      <c r="E629" s="5" t="n"/>
+    </row>
+    <row r="630">
+      <c r="A630" s="6" t="n"/>
+      <c r="B630" s="5" t="n"/>
+      <c r="C630" s="7" t="n"/>
+      <c r="D630" s="7" t="n"/>
+      <c r="E630" s="5" t="n"/>
+    </row>
+    <row r="631">
+      <c r="A631" s="6" t="n"/>
+      <c r="B631" s="5" t="n"/>
+      <c r="C631" s="7" t="n"/>
+      <c r="D631" s="7" t="n"/>
+      <c r="E631" s="5" t="n"/>
+    </row>
+    <row r="632">
+      <c r="A632" s="6" t="n"/>
+      <c r="B632" s="5" t="n"/>
+      <c r="C632" s="7" t="n"/>
+      <c r="D632" s="7" t="n"/>
+      <c r="E632" s="5" t="n"/>
+    </row>
+    <row r="633">
+      <c r="A633" s="6" t="n"/>
+      <c r="B633" s="5" t="n"/>
+      <c r="C633" s="7" t="n"/>
+      <c r="D633" s="7" t="n"/>
+      <c r="E633" s="5" t="n"/>
+    </row>
+    <row r="634">
+      <c r="A634" s="6" t="n"/>
+      <c r="B634" s="5" t="n"/>
+      <c r="C634" s="7" t="n"/>
+      <c r="D634" s="7" t="n"/>
+      <c r="E634" s="5" t="n"/>
+    </row>
+    <row r="635">
+      <c r="A635" s="6" t="n"/>
+      <c r="B635" s="5" t="n"/>
+      <c r="C635" s="7" t="n"/>
+      <c r="D635" s="7" t="n"/>
+      <c r="E635" s="5" t="n"/>
+    </row>
+    <row r="636">
+      <c r="A636" s="6" t="n"/>
+      <c r="B636" s="5" t="n"/>
+      <c r="C636" s="7" t="n"/>
+      <c r="D636" s="7" t="n"/>
+      <c r="E636" s="5" t="n"/>
+    </row>
+    <row r="637">
+      <c r="A637" s="6" t="n"/>
+      <c r="B637" s="5" t="n"/>
+      <c r="C637" s="7" t="n"/>
+      <c r="D637" s="7" t="n"/>
+      <c r="E637" s="5" t="n"/>
+    </row>
+    <row r="638">
+      <c r="A638" s="6" t="n"/>
+      <c r="B638" s="5" t="n"/>
+      <c r="C638" s="7" t="n"/>
+      <c r="D638" s="7" t="n"/>
+      <c r="E638" s="5" t="n"/>
+    </row>
+    <row r="639">
+      <c r="A639" s="6" t="n"/>
+      <c r="B639" s="5" t="n"/>
+      <c r="C639" s="7" t="n"/>
+      <c r="D639" s="7" t="n"/>
+      <c r="E639" s="5" t="n"/>
+    </row>
+    <row r="640">
+      <c r="A640" s="6" t="n"/>
+      <c r="B640" s="5" t="n"/>
+      <c r="C640" s="7" t="n"/>
+      <c r="D640" s="7" t="n"/>
+      <c r="E640" s="5" t="n"/>
+    </row>
+    <row r="641">
+      <c r="A641" s="6" t="n"/>
+      <c r="B641" s="5" t="n"/>
+      <c r="C641" s="7" t="n"/>
+      <c r="D641" s="7" t="n"/>
+      <c r="E641" s="5" t="n"/>
+    </row>
+    <row r="642">
+      <c r="A642" s="6" t="n"/>
+      <c r="B642" s="5" t="n"/>
+      <c r="C642" s="7" t="n"/>
+      <c r="D642" s="7" t="n"/>
+      <c r="E642" s="5" t="n"/>
+    </row>
+    <row r="643">
+      <c r="A643" s="6" t="n"/>
+      <c r="B643" s="5" t="n"/>
+      <c r="C643" s="7" t="n"/>
+      <c r="D643" s="7" t="n"/>
+      <c r="E643" s="5" t="n"/>
+    </row>
+    <row r="644">
+      <c r="A644" s="6" t="n"/>
+      <c r="B644" s="5" t="n"/>
+      <c r="C644" s="7" t="n"/>
+      <c r="D644" s="7" t="n"/>
+      <c r="E644" s="5" t="n"/>
+    </row>
+    <row r="645">
+      <c r="A645" s="6" t="n"/>
+      <c r="B645" s="5" t="n"/>
+      <c r="C645" s="7" t="n"/>
+      <c r="D645" s="7" t="n"/>
+      <c r="E645" s="5" t="n"/>
+    </row>
+    <row r="646">
+      <c r="A646" s="6" t="n"/>
+      <c r="B646" s="5" t="n"/>
+      <c r="C646" s="7" t="n"/>
+      <c r="D646" s="7" t="n"/>
+      <c r="E646" s="5" t="n"/>
+    </row>
+    <row r="647">
+      <c r="A647" s="6" t="n"/>
+      <c r="B647" s="5" t="n"/>
+      <c r="C647" s="7" t="n"/>
+      <c r="D647" s="7" t="n"/>
+      <c r="E647" s="5" t="n"/>
+    </row>
+    <row r="648">
+      <c r="A648" s="6" t="n"/>
+      <c r="B648" s="5" t="n"/>
+      <c r="C648" s="7" t="n"/>
+      <c r="D648" s="7" t="n"/>
+      <c r="E648" s="5" t="n"/>
+    </row>
+    <row r="649">
+      <c r="A649" s="6" t="n"/>
+      <c r="B649" s="5" t="n"/>
+      <c r="C649" s="7" t="n"/>
+      <c r="D649" s="7" t="n"/>
+      <c r="E649" s="5" t="n"/>
+    </row>
+    <row r="650">
+      <c r="A650" s="6" t="n"/>
+      <c r="B650" s="5" t="n"/>
+      <c r="C650" s="7" t="n"/>
+      <c r="D650" s="7" t="n"/>
+      <c r="E650" s="5" t="n"/>
+    </row>
+    <row r="651">
+      <c r="A651" s="6" t="n"/>
+      <c r="B651" s="5" t="n"/>
+      <c r="C651" s="7" t="n"/>
+      <c r="D651" s="7" t="n"/>
+      <c r="E651" s="5" t="n"/>
+    </row>
+    <row r="652">
+      <c r="A652" s="6" t="n"/>
+      <c r="B652" s="5" t="n"/>
+      <c r="C652" s="7" t="n"/>
+      <c r="D652" s="7" t="n"/>
+      <c r="E652" s="5" t="n"/>
+    </row>
+    <row r="653">
+      <c r="A653" s="6" t="n"/>
+      <c r="B653" s="5" t="n"/>
+      <c r="C653" s="7" t="n"/>
+      <c r="D653" s="7" t="n"/>
+      <c r="E653" s="5" t="n"/>
+    </row>
+    <row r="654">
+      <c r="A654" s="6" t="n"/>
+      <c r="B654" s="5" t="n"/>
+      <c r="C654" s="7" t="n"/>
+      <c r="D654" s="7" t="n"/>
+      <c r="E654" s="5" t="n"/>
+    </row>
+    <row r="655">
+      <c r="A655" s="6" t="n"/>
+      <c r="B655" s="5" t="n"/>
+      <c r="C655" s="7" t="n"/>
+      <c r="D655" s="7" t="n"/>
+      <c r="E655" s="5" t="n"/>
+    </row>
+    <row r="656">
+      <c r="A656" s="6" t="n"/>
+      <c r="B656" s="5" t="n"/>
+      <c r="C656" s="7" t="n"/>
+      <c r="D656" s="7" t="n"/>
+      <c r="E656" s="5" t="n"/>
+    </row>
+    <row r="657">
+      <c r="A657" s="6" t="n"/>
+      <c r="B657" s="5" t="n"/>
+      <c r="C657" s="7" t="n"/>
+      <c r="D657" s="7" t="n"/>
+      <c r="E657" s="5" t="n"/>
+    </row>
+    <row r="658">
+      <c r="A658" s="6" t="n"/>
+      <c r="B658" s="5" t="n"/>
+      <c r="C658" s="7" t="n"/>
+      <c r="D658" s="7" t="n"/>
+      <c r="E658" s="5" t="n"/>
+    </row>
+    <row r="659">
+      <c r="A659" s="6" t="n"/>
+      <c r="B659" s="5" t="n"/>
+      <c r="C659" s="7" t="n"/>
+      <c r="D659" s="7" t="n"/>
+      <c r="E659" s="5" t="n"/>
+    </row>
+    <row r="660">
+      <c r="A660" s="6" t="n"/>
+      <c r="B660" s="5" t="n"/>
+      <c r="C660" s="7" t="n"/>
+      <c r="D660" s="7" t="n"/>
+      <c r="E660" s="5" t="n"/>
+    </row>
+    <row r="661">
+      <c r="A661" s="6" t="n"/>
+      <c r="B661" s="5" t="n"/>
+      <c r="C661" s="7" t="n"/>
+      <c r="D661" s="7" t="n"/>
+      <c r="E661" s="5" t="n"/>
+    </row>
+    <row r="662">
+      <c r="A662" s="6" t="n"/>
+      <c r="B662" s="5" t="n"/>
+      <c r="C662" s="7" t="n"/>
+      <c r="D662" s="7" t="n"/>
+      <c r="E662" s="5" t="n"/>
+    </row>
+    <row r="663">
+      <c r="A663" s="6" t="n"/>
+      <c r="B663" s="5" t="n"/>
+      <c r="C663" s="7" t="n"/>
+      <c r="D663" s="7" t="n"/>
+      <c r="E663" s="5" t="n"/>
+    </row>
+    <row r="664">
+      <c r="A664" s="6" t="n"/>
+      <c r="B664" s="5" t="n"/>
+      <c r="C664" s="7" t="n"/>
+      <c r="D664" s="7" t="n"/>
+      <c r="E664" s="5" t="n"/>
+    </row>
+    <row r="665">
+      <c r="A665" s="6" t="n"/>
+      <c r="B665" s="5" t="n"/>
+      <c r="C665" s="7" t="n"/>
+      <c r="D665" s="7" t="n"/>
+      <c r="E665" s="5" t="n"/>
+    </row>
+    <row r="666">
+      <c r="A666" s="6" t="n"/>
+      <c r="B666" s="5" t="n"/>
+      <c r="C666" s="7" t="n"/>
+      <c r="D666" s="7" t="n"/>
+      <c r="E666" s="5" t="n"/>
+    </row>
+    <row r="667">
+      <c r="A667" s="6" t="n"/>
+      <c r="B667" s="5" t="n"/>
+      <c r="C667" s="7" t="n"/>
+      <c r="D667" s="7" t="n"/>
+      <c r="E667" s="5" t="n"/>
+    </row>
+    <row r="668">
+      <c r="A668" s="6" t="n"/>
+      <c r="B668" s="5" t="n"/>
+      <c r="C668" s="7" t="n"/>
+      <c r="D668" s="7" t="n"/>
+      <c r="E668" s="5" t="n"/>
+    </row>
+    <row r="669">
+      <c r="A669" s="6" t="n"/>
+      <c r="B669" s="5" t="n"/>
+      <c r="C669" s="7" t="n"/>
+      <c r="D669" s="7" t="n"/>
+      <c r="E669" s="5" t="n"/>
+    </row>
+    <row r="670">
+      <c r="A670" s="6" t="n"/>
+      <c r="B670" s="5" t="n"/>
+      <c r="C670" s="7" t="n"/>
+      <c r="D670" s="7" t="n"/>
+      <c r="E670" s="5" t="n"/>
+    </row>
+    <row r="671">
+      <c r="A671" s="6" t="n"/>
+      <c r="B671" s="5" t="n"/>
+      <c r="C671" s="7" t="n"/>
+      <c r="D671" s="7" t="n"/>
+      <c r="E671" s="5" t="n"/>
+    </row>
+    <row r="672">
+      <c r="A672" s="6" t="n"/>
+      <c r="B672" s="5" t="n"/>
+      <c r="C672" s="7" t="n"/>
+      <c r="D672" s="7" t="n"/>
+      <c r="E672" s="5" t="n"/>
+    </row>
+    <row r="673">
+      <c r="A673" s="6" t="n"/>
+      <c r="B673" s="5" t="n"/>
+      <c r="C673" s="7" t="n"/>
+      <c r="D673" s="7" t="n"/>
+      <c r="E673" s="5" t="n"/>
+    </row>
+    <row r="674">
+      <c r="A674" s="6" t="n"/>
+      <c r="B674" s="5" t="n"/>
+      <c r="C674" s="7" t="n"/>
+      <c r="D674" s="7" t="n"/>
+      <c r="E674" s="5" t="n"/>
+    </row>
+    <row r="675">
+      <c r="A675" s="6" t="n"/>
+      <c r="B675" s="5" t="n"/>
+      <c r="C675" s="7" t="n"/>
+      <c r="D675" s="7" t="n"/>
+      <c r="E675" s="5" t="n"/>
+    </row>
+    <row r="676">
+      <c r="A676" s="6" t="n"/>
+      <c r="B676" s="5" t="n"/>
+      <c r="C676" s="7" t="n"/>
+      <c r="D676" s="7" t="n"/>
+      <c r="E676" s="5" t="n"/>
+    </row>
+    <row r="677">
+      <c r="A677" s="6" t="n"/>
+      <c r="B677" s="5" t="n"/>
+      <c r="C677" s="7" t="n"/>
+      <c r="D677" s="7" t="n"/>
+      <c r="E677" s="5" t="n"/>
+    </row>
+    <row r="678">
+      <c r="A678" s="6" t="n"/>
+      <c r="B678" s="5" t="n"/>
+      <c r="C678" s="7" t="n"/>
+      <c r="D678" s="7" t="n"/>
+      <c r="E678" s="5" t="n"/>
+    </row>
+    <row r="679">
+      <c r="A679" s="6" t="n"/>
+      <c r="B679" s="5" t="n"/>
+      <c r="C679" s="7" t="n"/>
+      <c r="D679" s="7" t="n"/>
+      <c r="E679" s="5" t="n"/>
+    </row>
+    <row r="680">
+      <c r="A680" s="6" t="n"/>
+      <c r="B680" s="5" t="n"/>
+      <c r="C680" s="7" t="n"/>
+      <c r="D680" s="7" t="n"/>
+      <c r="E680" s="5" t="n"/>
+    </row>
+    <row r="681">
+      <c r="A681" s="6" t="n"/>
+      <c r="B681" s="5" t="n"/>
+      <c r="C681" s="7" t="n"/>
+      <c r="D681" s="7" t="n"/>
+      <c r="E681" s="5" t="n"/>
+    </row>
+    <row r="682">
+      <c r="A682" s="6" t="n"/>
+      <c r="B682" s="5" t="n"/>
+      <c r="C682" s="7" t="n"/>
+      <c r="D682" s="7" t="n"/>
+      <c r="E682" s="5" t="n"/>
+    </row>
+    <row r="683">
+      <c r="A683" s="6" t="n"/>
+      <c r="B683" s="5" t="n"/>
+      <c r="C683" s="7" t="n"/>
+      <c r="D683" s="7" t="n"/>
+      <c r="E683" s="5" t="n"/>
+    </row>
+    <row r="684">
+      <c r="A684" s="6" t="n"/>
+      <c r="B684" s="5" t="n"/>
+      <c r="C684" s="7" t="n"/>
+      <c r="D684" s="7" t="n"/>
+      <c r="E684" s="5" t="n"/>
+    </row>
+    <row r="685">
+      <c r="A685" s="6" t="n"/>
+      <c r="B685" s="5" t="n"/>
+      <c r="C685" s="7" t="n"/>
+      <c r="D685" s="7" t="n"/>
+      <c r="E685" s="5" t="n"/>
+    </row>
+    <row r="686">
+      <c r="A686" s="6" t="n"/>
+      <c r="B686" s="5" t="n"/>
+      <c r="C686" s="7" t="n"/>
+      <c r="D686" s="7" t="n"/>
+      <c r="E686" s="5" t="n"/>
+    </row>
+    <row r="687">
+      <c r="A687" s="6" t="n"/>
+      <c r="B687" s="5" t="n"/>
+      <c r="C687" s="7" t="n"/>
+      <c r="D687" s="7" t="n"/>
+      <c r="E687" s="5" t="n"/>
+    </row>
+    <row r="688">
+      <c r="A688" s="6" t="n"/>
+      <c r="B688" s="5" t="n"/>
+      <c r="C688" s="7" t="n"/>
+      <c r="D688" s="7" t="n"/>
+      <c r="E688" s="5" t="n"/>
+    </row>
+    <row r="689">
+      <c r="A689" s="6" t="n"/>
+      <c r="B689" s="5" t="n"/>
+      <c r="C689" s="7" t="n"/>
+      <c r="D689" s="7" t="n"/>
+      <c r="E689" s="5" t="n"/>
+    </row>
+    <row r="690">
+      <c r="A690" s="6" t="n"/>
+      <c r="B690" s="5" t="n"/>
+      <c r="C690" s="7" t="n"/>
+      <c r="D690" s="7" t="n"/>
+      <c r="E690" s="5" t="n"/>
+    </row>
+    <row r="691">
+      <c r="A691" s="6" t="n"/>
+      <c r="B691" s="5" t="n"/>
+      <c r="C691" s="7" t="n"/>
+      <c r="D691" s="7" t="n"/>
+      <c r="E691" s="5" t="n"/>
+    </row>
+    <row r="692">
+      <c r="A692" s="6" t="n"/>
+      <c r="B692" s="5" t="n"/>
+      <c r="C692" s="7" t="n"/>
+      <c r="D692" s="7" t="n"/>
+      <c r="E692" s="5" t="n"/>
+    </row>
+    <row r="693">
+      <c r="A693" s="6" t="n"/>
+      <c r="B693" s="5" t="n"/>
+      <c r="C693" s="7" t="n"/>
+      <c r="D693" s="7" t="n"/>
+      <c r="E693" s="5" t="n"/>
+    </row>
+    <row r="694">
+      <c r="A694" s="6" t="n"/>
+      <c r="B694" s="5" t="n"/>
+      <c r="C694" s="7" t="n"/>
+      <c r="D694" s="7" t="n"/>
+      <c r="E694" s="5" t="n"/>
+    </row>
+    <row r="695">
+      <c r="A695" s="6" t="n"/>
+      <c r="B695" s="5" t="n"/>
+      <c r="C695" s="7" t="n"/>
+      <c r="D695" s="7" t="n"/>
+      <c r="E695" s="5" t="n"/>
+    </row>
+    <row r="696">
+      <c r="A696" s="6" t="n"/>
+      <c r="B696" s="5" t="n"/>
+      <c r="C696" s="7" t="n"/>
+      <c r="D696" s="7" t="n"/>
+      <c r="E696" s="5" t="n"/>
+    </row>
+    <row r="697">
+      <c r="A697" s="6" t="n"/>
+      <c r="B697" s="5" t="n"/>
+      <c r="C697" s="7" t="n"/>
+      <c r="D697" s="7" t="n"/>
+      <c r="E697" s="5" t="n"/>
+    </row>
+    <row r="698">
+      <c r="A698" s="6" t="n"/>
+      <c r="B698" s="5" t="n"/>
+      <c r="C698" s="7" t="n"/>
+      <c r="D698" s="7" t="n"/>
+      <c r="E698" s="5" t="n"/>
+    </row>
+    <row r="699">
+      <c r="A699" s="6" t="n"/>
+      <c r="B699" s="5" t="n"/>
+      <c r="C699" s="7" t="n"/>
+      <c r="D699" s="7" t="n"/>
+      <c r="E699" s="5" t="n"/>
+    </row>
+    <row r="700">
+      <c r="A700" s="6" t="n"/>
+      <c r="B700" s="5" t="n"/>
+      <c r="C700" s="7" t="n"/>
+      <c r="D700" s="7" t="n"/>
+      <c r="E700" s="5" t="n"/>
+    </row>
+    <row r="701">
+      <c r="A701" s="6" t="n"/>
+      <c r="B701" s="5" t="n"/>
+      <c r="C701" s="7" t="n"/>
+      <c r="D701" s="7" t="n"/>
+      <c r="E701" s="5" t="n"/>
+    </row>
+    <row r="702">
+      <c r="A702" s="6" t="n"/>
+      <c r="B702" s="5" t="n"/>
+      <c r="C702" s="7" t="n"/>
+      <c r="D702" s="7" t="n"/>
+      <c r="E702" s="5" t="n"/>
+    </row>
+    <row r="703">
+      <c r="A703" s="6" t="n"/>
+      <c r="B703" s="5" t="n"/>
+      <c r="C703" s="7" t="n"/>
+      <c r="D703" s="7" t="n"/>
+      <c r="E703" s="5" t="n"/>
+    </row>
+    <row r="704">
+      <c r="A704" s="6" t="n"/>
+      <c r="B704" s="5" t="n"/>
+      <c r="C704" s="7" t="n"/>
+      <c r="D704" s="7" t="n"/>
+      <c r="E704" s="5" t="n"/>
+    </row>
+    <row r="705">
+      <c r="A705" s="6" t="n"/>
+      <c r="B705" s="5" t="n"/>
+      <c r="C705" s="7" t="n"/>
+      <c r="D705" s="7" t="n"/>
+      <c r="E705" s="5" t="n"/>
+    </row>
+    <row r="706">
+      <c r="A706" s="6" t="n"/>
+      <c r="B706" s="5" t="n"/>
+      <c r="C706" s="7" t="n"/>
+      <c r="D706" s="7" t="n"/>
+      <c r="E706" s="5" t="n"/>
+    </row>
+    <row r="707">
+      <c r="A707" s="6" t="n"/>
+      <c r="B707" s="5" t="n"/>
+      <c r="C707" s="7" t="n"/>
+      <c r="D707" s="7" t="n"/>
+      <c r="E707" s="5" t="n"/>
+    </row>
+    <row r="708">
+      <c r="A708" s="6" t="n"/>
+      <c r="B708" s="5" t="n"/>
+      <c r="C708" s="7" t="n"/>
+      <c r="D708" s="7" t="n"/>
+      <c r="E708" s="5" t="n"/>
+    </row>
+    <row r="709">
+      <c r="A709" s="6" t="n"/>
+      <c r="B709" s="5" t="n"/>
+      <c r="C709" s="7" t="n"/>
+      <c r="D709" s="7" t="n"/>
+      <c r="E709" s="5" t="n"/>
+    </row>
+    <row r="710">
+      <c r="A710" s="6" t="n"/>
+      <c r="B710" s="5" t="n"/>
+      <c r="C710" s="7" t="n"/>
+      <c r="D710" s="7" t="n"/>
+      <c r="E710" s="5" t="n"/>
+    </row>
+    <row r="711">
+      <c r="A711" s="6" t="n"/>
+      <c r="B711" s="5" t="n"/>
+      <c r="C711" s="7" t="n"/>
+      <c r="D711" s="7" t="n"/>
+      <c r="E711" s="5" t="n"/>
+    </row>
+    <row r="712">
+      <c r="A712" s="6" t="n"/>
+      <c r="B712" s="5" t="n"/>
+      <c r="C712" s="7" t="n"/>
+      <c r="D712" s="7" t="n"/>
+      <c r="E712" s="5" t="n"/>
+    </row>
+    <row r="713">
+      <c r="A713" s="6" t="n"/>
+      <c r="B713" s="5" t="n"/>
+      <c r="C713" s="7" t="n"/>
+      <c r="D713" s="7" t="n"/>
+      <c r="E713" s="5" t="n"/>
+    </row>
+    <row r="714">
+      <c r="A714" s="6" t="n"/>
+      <c r="B714" s="5" t="n"/>
+      <c r="C714" s="7" t="n"/>
+      <c r="D714" s="7" t="n"/>
+      <c r="E714" s="5" t="n"/>
+    </row>
+    <row r="715">
+      <c r="A715" s="6" t="n"/>
+      <c r="B715" s="5" t="n"/>
+      <c r="C715" s="7" t="n"/>
+      <c r="D715" s="7" t="n"/>
+      <c r="E715" s="5" t="n"/>
+    </row>
+    <row r="716">
+      <c r="A716" s="6" t="n"/>
+      <c r="B716" s="5" t="n"/>
+      <c r="C716" s="7" t="n"/>
+      <c r="D716" s="7" t="n"/>
+      <c r="E716" s="5" t="n"/>
+    </row>
+    <row r="717">
+      <c r="A717" s="6" t="n"/>
+      <c r="B717" s="5" t="n"/>
+      <c r="C717" s="7" t="n"/>
+      <c r="D717" s="7" t="n"/>
+      <c r="E717" s="5" t="n"/>
+    </row>
+    <row r="718">
+      <c r="A718" s="6" t="n"/>
+      <c r="B718" s="5" t="n"/>
+      <c r="C718" s="7" t="n"/>
+      <c r="D718" s="7" t="n"/>
+      <c r="E718" s="5" t="n"/>
+    </row>
+    <row r="719">
+      <c r="A719" s="6" t="n"/>
+      <c r="B719" s="5" t="n"/>
+      <c r="C719" s="7" t="n"/>
+      <c r="D719" s="7" t="n"/>
+      <c r="E719" s="5" t="n"/>
+    </row>
+    <row r="720">
+      <c r="A720" s="6" t="n"/>
+      <c r="B720" s="5" t="n"/>
+      <c r="C720" s="7" t="n"/>
+      <c r="D720" s="7" t="n"/>
+      <c r="E720" s="5" t="n"/>
+    </row>
+    <row r="721">
+      <c r="A721" s="6" t="n"/>
+      <c r="B721" s="5" t="n"/>
+      <c r="C721" s="7" t="n"/>
+      <c r="D721" s="7" t="n"/>
+      <c r="E721" s="5" t="n"/>
+    </row>
+    <row r="722">
+      <c r="A722" s="6" t="n"/>
+      <c r="B722" s="5" t="n"/>
+      <c r="C722" s="7" t="n"/>
+      <c r="D722" s="7" t="n"/>
+      <c r="E722" s="5" t="n"/>
+    </row>
+    <row r="723">
+      <c r="A723" s="6" t="n"/>
+      <c r="B723" s="5" t="n"/>
+      <c r="C723" s="7" t="n"/>
+      <c r="D723" s="7" t="n"/>
+      <c r="E723" s="5" t="n"/>
+    </row>
+    <row r="724">
+      <c r="A724" s="6" t="n"/>
+      <c r="B724" s="5" t="n"/>
+      <c r="C724" s="7" t="n"/>
+      <c r="D724" s="7" t="n"/>
+      <c r="E724" s="5" t="n"/>
+    </row>
+    <row r="725">
+      <c r="A725" s="6" t="n"/>
+      <c r="B725" s="5" t="n"/>
+      <c r="C725" s="7" t="n"/>
+      <c r="D725" s="7" t="n"/>
+      <c r="E725" s="5" t="n"/>
+    </row>
+    <row r="726">
+      <c r="A726" s="6" t="n"/>
+      <c r="B726" s="5" t="n"/>
+      <c r="C726" s="7" t="n"/>
+      <c r="D726" s="7" t="n"/>
+      <c r="E726" s="5" t="n"/>
+    </row>
+    <row r="727">
+      <c r="A727" s="6" t="n"/>
+      <c r="B727" s="5" t="n"/>
+      <c r="C727" s="7" t="n"/>
+      <c r="D727" s="7" t="n"/>
+      <c r="E727" s="5" t="n"/>
+    </row>
+    <row r="728">
+      <c r="A728" s="6" t="n"/>
+      <c r="B728" s="5" t="n"/>
+      <c r="C728" s="7" t="n"/>
+      <c r="D728" s="7" t="n"/>
+      <c r="E728" s="5" t="n"/>
+    </row>
+    <row r="729">
+      <c r="A729" s="6" t="n"/>
+      <c r="B729" s="5" t="n"/>
+      <c r="C729" s="7" t="n"/>
+      <c r="D729" s="7" t="n"/>
+      <c r="E729" s="5" t="n"/>
+    </row>
+    <row r="730">
+      <c r="A730" s="6" t="n"/>
+      <c r="B730" s="5" t="n"/>
+      <c r="C730" s="7" t="n"/>
+      <c r="D730" s="7" t="n"/>
+      <c r="E730" s="5" t="n"/>
+    </row>
+    <row r="731">
+      <c r="A731" s="6" t="n"/>
+      <c r="B731" s="5" t="n"/>
+      <c r="C731" s="7" t="n"/>
+      <c r="D731" s="7" t="n"/>
+      <c r="E731" s="5" t="n"/>
+    </row>
+    <row r="732">
+      <c r="A732" s="6" t="n"/>
+      <c r="B732" s="5" t="n"/>
+      <c r="C732" s="7" t="n"/>
+      <c r="D732" s="7" t="n"/>
+      <c r="E732" s="5" t="n"/>
+    </row>
+    <row r="733">
+      <c r="A733" s="6" t="n"/>
+      <c r="B733" s="5" t="n"/>
+      <c r="C733" s="7" t="n"/>
+      <c r="D733" s="7" t="n"/>
+      <c r="E733" s="5" t="n"/>
+    </row>
+    <row r="734">
+      <c r="A734" s="6" t="n"/>
+      <c r="B734" s="5" t="n"/>
+      <c r="C734" s="7" t="n"/>
+      <c r="D734" s="7" t="n"/>
+      <c r="E734" s="5" t="n"/>
+    </row>
+    <row r="735">
+      <c r="A735" s="6" t="n"/>
+      <c r="B735" s="5" t="n"/>
+      <c r="C735" s="7" t="n"/>
+      <c r="D735" s="7" t="n"/>
+      <c r="E735" s="5" t="n"/>
+    </row>
+    <row r="736">
+      <c r="A736" s="6" t="n"/>
+      <c r="B736" s="5" t="n"/>
+      <c r="C736" s="7" t="n"/>
+      <c r="D736" s="7" t="n"/>
+      <c r="E736" s="5" t="n"/>
+    </row>
+    <row r="737">
+      <c r="A737" s="6" t="n"/>
+      <c r="B737" s="5" t="n"/>
+      <c r="C737" s="7" t="n"/>
+      <c r="D737" s="7" t="n"/>
+      <c r="E737" s="5" t="n"/>
+    </row>
+    <row r="738">
+      <c r="A738" s="6" t="n"/>
+      <c r="B738" s="5" t="n"/>
+      <c r="C738" s="7" t="n"/>
+      <c r="D738" s="7" t="n"/>
+      <c r="E738" s="5" t="n"/>
+    </row>
+    <row r="739">
+      <c r="A739" s="6" t="n"/>
+      <c r="B739" s="5" t="n"/>
+      <c r="C739" s="7" t="n"/>
+      <c r="D739" s="7" t="n"/>
+      <c r="E739" s="5" t="n"/>
+    </row>
+    <row r="740">
+      <c r="A740" s="6" t="n"/>
+      <c r="B740" s="5" t="n"/>
+      <c r="C740" s="7" t="n"/>
+      <c r="D740" s="7" t="n"/>
+      <c r="E740" s="5" t="n"/>
+    </row>
+    <row r="741">
+      <c r="A741" s="6" t="n"/>
+      <c r="B741" s="5" t="n"/>
+      <c r="C741" s="7" t="n"/>
+      <c r="D741" s="7" t="n"/>
+      <c r="E741" s="5" t="n"/>
+    </row>
+    <row r="742">
+      <c r="A742" s="6" t="n"/>
+      <c r="B742" s="5" t="n"/>
+      <c r="C742" s="7" t="n"/>
+      <c r="D742" s="7" t="n"/>
+      <c r="E742" s="5" t="n"/>
+    </row>
+    <row r="743">
+      <c r="A743" s="6" t="n"/>
+      <c r="B743" s="5" t="n"/>
+      <c r="C743" s="7" t="n"/>
+      <c r="D743" s="7" t="n"/>
+      <c r="E743" s="5" t="n"/>
+    </row>
+    <row r="744">
+      <c r="A744" s="6" t="n"/>
+      <c r="B744" s="5" t="n"/>
+      <c r="C744" s="7" t="n"/>
+      <c r="D744" s="7" t="n"/>
+      <c r="E744" s="5" t="n"/>
+    </row>
+    <row r="745">
+      <c r="A745" s="6" t="n"/>
+      <c r="B745" s="5" t="n"/>
+      <c r="C745" s="7" t="n"/>
+      <c r="D745" s="7" t="n"/>
+      <c r="E745" s="5" t="n"/>
+    </row>
+    <row r="746">
+      <c r="A746" s="6" t="n"/>
+      <c r="B746" s="5" t="n"/>
+      <c r="C746" s="7" t="n"/>
+      <c r="D746" s="7" t="n"/>
+      <c r="E746" s="5" t="n"/>
+    </row>
+    <row r="747">
+      <c r="A747" s="6" t="n"/>
+      <c r="B747" s="5" t="n"/>
+      <c r="C747" s="7" t="n"/>
+      <c r="D747" s="7" t="n"/>
+      <c r="E747" s="5" t="n"/>
+    </row>
+    <row r="748">
+      <c r="A748" s="6" t="n"/>
+      <c r="B748" s="5" t="n"/>
+      <c r="C748" s="7" t="n"/>
+      <c r="D748" s="7" t="n"/>
+      <c r="E748" s="5" t="n"/>
+    </row>
+    <row r="749">
+      <c r="A749" s="6" t="n"/>
+      <c r="B749" s="5" t="n"/>
+      <c r="C749" s="7" t="n"/>
+      <c r="D749" s="7" t="n"/>
+      <c r="E749" s="5" t="n"/>
+    </row>
+    <row r="750">
+      <c r="A750" s="6" t="n"/>
+      <c r="B750" s="5" t="n"/>
+      <c r="C750" s="7" t="n"/>
+      <c r="D750" s="7" t="n"/>
+      <c r="E750" s="5" t="n"/>
+    </row>
+    <row r="751">
+      <c r="A751" s="6" t="n"/>
+      <c r="B751" s="5" t="n"/>
+      <c r="C751" s="7" t="n"/>
+      <c r="D751" s="7" t="n"/>
+      <c r="E751" s="5" t="n"/>
+    </row>
+    <row r="752">
+      <c r="A752" s="6" t="n"/>
+      <c r="B752" s="5" t="n"/>
+      <c r="C752" s="7" t="n"/>
+      <c r="D752" s="7" t="n"/>
+      <c r="E752" s="5" t="n"/>
+    </row>
+    <row r="753">
+      <c r="A753" s="6" t="n"/>
+      <c r="B753" s="5" t="n"/>
+      <c r="C753" s="7" t="n"/>
+      <c r="D753" s="7" t="n"/>
+      <c r="E753" s="5" t="n"/>
+    </row>
+    <row r="754">
+      <c r="A754" s="6" t="n"/>
+      <c r="B754" s="5" t="n"/>
+      <c r="C754" s="7" t="n"/>
+      <c r="D754" s="7" t="n"/>
+      <c r="E754" s="5" t="n"/>
+    </row>
+    <row r="755">
+      <c r="A755" s="6" t="n"/>
+      <c r="B755" s="5" t="n"/>
+      <c r="C755" s="7" t="n"/>
+      <c r="D755" s="7" t="n"/>
+      <c r="E755" s="5" t="n"/>
+    </row>
+    <row r="756">
+      <c r="A756" s="6" t="n"/>
+      <c r="B756" s="5" t="n"/>
+      <c r="C756" s="7" t="n"/>
+      <c r="D756" s="7" t="n"/>
+      <c r="E756" s="5" t="n"/>
+    </row>
+    <row r="757">
+      <c r="A757" s="6" t="n"/>
+      <c r="B757" s="5" t="n"/>
+      <c r="C757" s="7" t="n"/>
+      <c r="D757" s="7" t="n"/>
+      <c r="E757" s="5" t="n"/>
+    </row>
+    <row r="758">
+      <c r="A758" s="6" t="n"/>
+      <c r="B758" s="5" t="n"/>
+      <c r="C758" s="7" t="n"/>
+      <c r="D758" s="7" t="n"/>
+      <c r="E758" s="5" t="n"/>
+    </row>
+    <row r="759">
+      <c r="A759" s="6" t="n"/>
+      <c r="B759" s="5" t="n"/>
+      <c r="C759" s="7" t="n"/>
+      <c r="D759" s="7" t="n"/>
+      <c r="E759" s="5" t="n"/>
+    </row>
+    <row r="760">
+      <c r="A760" s="6" t="n"/>
+      <c r="B760" s="5" t="n"/>
+      <c r="C760" s="7" t="n"/>
+      <c r="D760" s="7" t="n"/>
+      <c r="E760" s="5" t="n"/>
+    </row>
+    <row r="761">
+      <c r="A761" s="6" t="n"/>
+      <c r="B761" s="5" t="n"/>
+      <c r="C761" s="7" t="n"/>
+      <c r="D761" s="7" t="n"/>
+      <c r="E761" s="5" t="n"/>
+    </row>
+    <row r="762">
+      <c r="A762" s="6" t="n"/>
+      <c r="B762" s="5" t="n"/>
+      <c r="C762" s="7" t="n"/>
+      <c r="D762" s="7" t="n"/>
+      <c r="E762" s="5" t="n"/>
+    </row>
+    <row r="763">
+      <c r="A763" s="6" t="n"/>
+      <c r="B763" s="5" t="n"/>
+      <c r="C763" s="7" t="n"/>
+      <c r="D763" s="7" t="n"/>
+      <c r="E763" s="5" t="n"/>
+    </row>
+    <row r="764">
+      <c r="A764" s="6" t="n"/>
+      <c r="B764" s="5" t="n"/>
+      <c r="C764" s="7" t="n"/>
+      <c r="D764" s="7" t="n"/>
+      <c r="E764" s="5" t="n"/>
+    </row>
+    <row r="765">
+      <c r="A765" s="6" t="n"/>
+      <c r="B765" s="5" t="n"/>
+      <c r="C765" s="7" t="n"/>
+      <c r="D765" s="7" t="n"/>
+      <c r="E765" s="5" t="n"/>
+    </row>
+    <row r="766">
+      <c r="A766" s="6" t="n"/>
+      <c r="B766" s="5" t="n"/>
+      <c r="C766" s="7" t="n"/>
+      <c r="D766" s="7" t="n"/>
+      <c r="E766" s="5" t="n"/>
+    </row>
+    <row r="767">
+      <c r="A767" s="6" t="n"/>
+      <c r="B767" s="5" t="n"/>
+      <c r="C767" s="7" t="n"/>
+      <c r="D767" s="7" t="n"/>
+      <c r="E767" s="5" t="n"/>
+    </row>
+    <row r="768">
+      <c r="A768" s="6" t="n"/>
+      <c r="B768" s="5" t="n"/>
+      <c r="C768" s="7" t="n"/>
+      <c r="D768" s="7" t="n"/>
+      <c r="E768" s="5" t="n"/>
+    </row>
+    <row r="769">
+      <c r="A769" s="6" t="n"/>
+      <c r="B769" s="5" t="n"/>
+      <c r="C769" s="7" t="n"/>
+      <c r="D769" s="7" t="n"/>
+      <c r="E769" s="5" t="n"/>
+    </row>
+    <row r="770">
+      <c r="A770" s="6" t="n"/>
+      <c r="B770" s="5" t="n"/>
+      <c r="C770" s="7" t="n"/>
+      <c r="D770" s="7" t="n"/>
+      <c r="E770" s="5" t="n"/>
+    </row>
+    <row r="771">
+      <c r="A771" s="6" t="n"/>
+      <c r="B771" s="5" t="n"/>
+      <c r="C771" s="7" t="n"/>
+      <c r="D771" s="7" t="n"/>
+      <c r="E771" s="5" t="n"/>
+    </row>
+    <row r="772">
+      <c r="A772" s="6" t="n"/>
+      <c r="B772" s="5" t="n"/>
+      <c r="C772" s="7" t="n"/>
+      <c r="D772" s="7" t="n"/>
+      <c r="E772" s="5" t="n"/>
+    </row>
+    <row r="773">
+      <c r="A773" s="6" t="n"/>
+      <c r="B773" s="5" t="n"/>
+      <c r="C773" s="7" t="n"/>
+      <c r="D773" s="7" t="n"/>
+      <c r="E773" s="5" t="n"/>
+    </row>
+    <row r="774">
+      <c r="A774" s="6" t="n"/>
+      <c r="B774" s="5" t="n"/>
+      <c r="C774" s="7" t="n"/>
+      <c r="D774" s="7" t="n"/>
+      <c r="E774" s="5" t="n"/>
+    </row>
+    <row r="775">
+      <c r="A775" s="6" t="n"/>
+      <c r="B775" s="5" t="n"/>
+      <c r="C775" s="7" t="n"/>
+      <c r="D775" s="7" t="n"/>
+      <c r="E775" s="5" t="n"/>
+    </row>
+    <row r="776">
+      <c r="A776" s="6" t="n"/>
+      <c r="B776" s="5" t="n"/>
+      <c r="C776" s="7" t="n"/>
+      <c r="D776" s="7" t="n"/>
+      <c r="E776" s="5" t="n"/>
+    </row>
+    <row r="777">
+      <c r="A777" s="6" t="n"/>
+      <c r="B777" s="5" t="n"/>
+      <c r="C777" s="7" t="n"/>
+      <c r="D777" s="7" t="n"/>
+      <c r="E777" s="5" t="n"/>
+    </row>
+    <row r="778">
+      <c r="A778" s="6" t="n"/>
+      <c r="B778" s="5" t="n"/>
+      <c r="C778" s="7" t="n"/>
+      <c r="D778" s="7" t="n"/>
+      <c r="E778" s="5" t="n"/>
+    </row>
+    <row r="779">
+      <c r="A779" s="6" t="n"/>
+      <c r="B779" s="5" t="n"/>
+      <c r="C779" s="7" t="n"/>
+      <c r="D779" s="7" t="n"/>
+      <c r="E779" s="5" t="n"/>
+    </row>
+    <row r="780">
+      <c r="A780" s="6" t="n"/>
+      <c r="B780" s="5" t="n"/>
+      <c r="C780" s="7" t="n"/>
+      <c r="D780" s="7" t="n"/>
+      <c r="E780" s="5" t="n"/>
+    </row>
+    <row r="781">
+      <c r="A781" s="6" t="n"/>
+      <c r="B781" s="5" t="n"/>
+      <c r="C781" s="7" t="n"/>
+      <c r="D781" s="7" t="n"/>
+      <c r="E781" s="5" t="n"/>
+    </row>
+    <row r="782">
+      <c r="A782" s="6" t="n"/>
+      <c r="B782" s="5" t="n"/>
+      <c r="C782" s="7" t="n"/>
+      <c r="D782" s="7" t="n"/>
+      <c r="E782" s="5" t="n"/>
+    </row>
+    <row r="783">
+      <c r="A783" s="6" t="n"/>
+      <c r="B783" s="5" t="n"/>
+      <c r="C783" s="7" t="n"/>
+      <c r="D783" s="7" t="n"/>
+      <c r="E783" s="5" t="n"/>
+    </row>
+    <row r="784">
+      <c r="A784" s="6" t="n"/>
+      <c r="B784" s="5" t="n"/>
+      <c r="C784" s="7" t="n"/>
+      <c r="D784" s="7" t="n"/>
+      <c r="E784" s="5" t="n"/>
+    </row>
+    <row r="785">
+      <c r="A785" s="6" t="n"/>
+      <c r="B785" s="5" t="n"/>
+      <c r="C785" s="7" t="n"/>
+      <c r="D785" s="7" t="n"/>
+      <c r="E785" s="5" t="n"/>
+    </row>
+    <row r="786">
+      <c r="A786" s="6" t="n"/>
+      <c r="B786" s="5" t="n"/>
+      <c r="C786" s="7" t="n"/>
+      <c r="D786" s="7" t="n"/>
+      <c r="E786" s="5" t="n"/>
+    </row>
+    <row r="787">
+      <c r="A787" s="6" t="n"/>
+      <c r="B787" s="5" t="n"/>
+      <c r="C787" s="7" t="n"/>
+      <c r="D787" s="7" t="n"/>
+      <c r="E787" s="5" t="n"/>
+    </row>
+    <row r="788">
+      <c r="A788" s="6" t="n"/>
+      <c r="B788" s="5" t="n"/>
+      <c r="C788" s="7" t="n"/>
+      <c r="D788" s="7" t="n"/>
+      <c r="E788" s="5" t="n"/>
+    </row>
+    <row r="789">
+      <c r="A789" s="6" t="n"/>
+      <c r="B789" s="5" t="n"/>
+      <c r="C789" s="7" t="n"/>
+      <c r="D789" s="7" t="n"/>
+      <c r="E789" s="5" t="n"/>
+    </row>
+    <row r="790">
+      <c r="A790" s="6" t="n"/>
+      <c r="B790" s="5" t="n"/>
+      <c r="C790" s="7" t="n"/>
+      <c r="D790" s="7" t="n"/>
+      <c r="E790" s="5" t="n"/>
+    </row>
+    <row r="791">
+      <c r="A791" s="6" t="n"/>
+      <c r="B791" s="5" t="n"/>
+      <c r="C791" s="7" t="n"/>
+      <c r="D791" s="7" t="n"/>
+      <c r="E791" s="5" t="n"/>
+    </row>
+    <row r="792">
+      <c r="A792" s="6" t="n"/>
+      <c r="B792" s="5" t="n"/>
+      <c r="C792" s="7" t="n"/>
+      <c r="D792" s="7" t="n"/>
+      <c r="E792" s="5" t="n"/>
+    </row>
+    <row r="793">
+      <c r="A793" s="6" t="n"/>
+      <c r="B793" s="5" t="n"/>
+      <c r="C793" s="7" t="n"/>
+      <c r="D793" s="7" t="n"/>
+      <c r="E793" s="5" t="n"/>
+    </row>
+    <row r="794">
+      <c r="A794" s="6" t="n"/>
+      <c r="B794" s="5" t="n"/>
+      <c r="C794" s="7" t="n"/>
+      <c r="D794" s="7" t="n"/>
+      <c r="E794" s="5" t="n"/>
+    </row>
+    <row r="795">
+      <c r="A795" s="6" t="n"/>
+      <c r="B795" s="5" t="n"/>
+      <c r="C795" s="7" t="n"/>
+      <c r="D795" s="7" t="n"/>
+      <c r="E795" s="5" t="n"/>
+    </row>
+    <row r="796">
+      <c r="A796" s="6" t="n"/>
+      <c r="B796" s="5" t="n"/>
+      <c r="C796" s="7" t="n"/>
+      <c r="D796" s="7" t="n"/>
+      <c r="E796" s="5" t="n"/>
+    </row>
+    <row r="797">
+      <c r="A797" s="6" t="n"/>
+      <c r="B797" s="5" t="n"/>
+      <c r="C797" s="7" t="n"/>
+      <c r="D797" s="7" t="n"/>
+      <c r="E797" s="5" t="n"/>
+    </row>
+    <row r="798">
+      <c r="A798" s="6" t="n"/>
+      <c r="B798" s="5" t="n"/>
+      <c r="C798" s="7" t="n"/>
+      <c r="D798" s="7" t="n"/>
+      <c r="E798" s="5" t="n"/>
+    </row>
+    <row r="799">
+      <c r="A799" s="6" t="n"/>
+      <c r="B799" s="5" t="n"/>
+      <c r="C799" s="7" t="n"/>
+      <c r="D799" s="7" t="n"/>
+      <c r="E799" s="5" t="n"/>
+    </row>
+    <row r="800">
+      <c r="A800" s="6" t="n"/>
+      <c r="B800" s="5" t="n"/>
+      <c r="C800" s="7" t="n"/>
+      <c r="D800" s="7" t="n"/>
+      <c r="E800" s="5" t="n"/>
+    </row>
+    <row r="801">
+      <c r="A801" s="6" t="n"/>
+      <c r="B801" s="5" t="n"/>
+      <c r="C801" s="7" t="n"/>
+      <c r="D801" s="7" t="n"/>
+      <c r="E801" s="5" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2 B3 B4 B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 B21 B22 B23 B24 B25 B26 B27 B28 B29 B30 B31 B32 B33 B34 B35 B36 B37 B38 B39 B40 B41 B42 B43 B44 B45 B46 B47 B48 B49 B50 B51 B52 B53 B54 B55 B56 B57 B58 B59 B60 B61 B62 B63 B64 B65 B66 B67 B68 B69 B70 B71 B72 B73 B74 B75 B76 B77 B78 B79 B80 B81 B82 B83 B84 B85 B86 B87 B88 B89 B90 B91 B92 B93 B94 B95 B96 B97 B98 B99 B100 B101 B102 B103 B104 B105 B106 B107 B108 B109 B110 B111 B112 B113 B114 B115 B116 B117 B118 B119 B120 B121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="店舗名エラー" error="店舗マスタの一覧にある店舗名を選択してください。" type="list">
+    <dataValidation sqref="B2 B3 B4 B5 B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 B21 B22 B23 B24 B25 B26 B27 B28 B29 B30 B31 B32 B33 B34 B35 B36 B37 B38 B39 B40 B41 B42 B43 B44 B45 B46 B47 B48 B49 B50 B51 B52 B53 B54 B55 B56 B57 B58 B59 B60 B61 B62 B63 B64 B65 B66 B67 B68 B69 B70 B71 B72 B73 B74 B75 B76 B77 B78 B79 B80 B81 B82 B83 B84 B85 B86 B87 B88 B89 B90 B91 B92 B93 B94 B95 B96 B97 B98 B99 B100 B101 B102 B103 B104 B105 B106 B107 B108 B109 B110 B111 B112 B113 B114 B115 B116 B117 B118 B119 B120 B121 B122 B123 B124 B125 B126 B127 B128 B129 B130 B131 B132 B133 B134 B135 B136 B137 B138 B139 B140 B141 B142 B143 B144 B145 B146 B147 B148 B149 B150 B151 B152 B153 B154 B155 B156 B157 B158 B159 B160 B161 B162 B163 B164 B165 B166 B167 B168 B169 B170 B171 B172 B173 B174 B175 B176 B177 B178 B179 B180 B181 B182 B183 B184 B185 B186 B187 B188 B189 B190 B191 B192 B193 B194 B195 B196 B197 B198 B199 B200 B201 B202 B203 B204 B205 B206 B207 B208 B209 B210 B211 B212 B213 B214 B215 B216 B217 B218 B219 B220 B221 B222 B223 B224 B225 B226 B227 B228 B229 B230 B231 B232 B233 B234 B235 B236 B237 B238 B239 B240 B241 B242 B243 B244 B245 B246 B247 B248 B249 B250 B251 B252 B253 B254 B255 B256 B257 B258 B259 B260 B261 B262 B263 B264 B265 B266 B267 B268 B269 B270 B271 B272 B273 B274 B275 B276 B277 B278 B279 B280 B281 B282 B283 B284 B285 B286 B287 B288 B289 B290 B291 B292 B293 B294 B295 B296 B297 B298 B299 B300 B301 B302 B303 B304 B305 B306 B307 B308 B309 B310 B311 B312 B313 B314 B315 B316 B317 B318 B319 B320 B321 B322 B323 B324 B325 B326 B327 B328 B329 B330 B331 B332 B333 B334 B335 B336 B337 B338 B339 B340 B341 B342 B343 B344 B345 B346 B347 B348 B349 B350 B351 B352 B353 B354 B355 B356 B357 B358 B359 B360 B361 B362 B363 B364 B365 B366 B367 B368 B369 B370 B371 B372 B373 B374 B375 B376 B377 B378 B379 B380 B381 B382 B383 B384 B385 B386 B387 B388 B389 B390 B391 B392 B393 B394 B395 B396 B397 B398 B399 B400 B401 B402 B403 B404 B405 B406 B407 B408 B409 B410 B411 B412 B413 B414 B415 B416 B417 B418 B419 B420 B421 B422 B423 B424 B425 B426 B427 B428 B429 B430 B431 B432 B433 B434 B435 B436 B437 B438 B439 B440 B441 B442 B443 B444 B445 B446 B447 B448 B449 B450 B451 B452 B453 B454 B455 B456 B457 B458 B459 B460 B461 B462 B463 B464 B465 B466 B467 B468 B469 B470 B471 B472 B473 B474 B475 B476 B477 B478 B479 B480 B481 B482 B483 B484 B485 B486 B487 B488 B489 B490 B491 B492 B493 B494 B495 B496 B497 B498 B499 B500 B501 B502 B503 B504 B505 B506 B507 B508 B509 B510 B511 B512 B513 B514 B515 B516 B517 B518 B519 B520 B521 B522 B523 B524 B525 B526 B527 B528 B529 B530 B531 B532 B533 B534 B535 B536 B537 B538 B539 B540 B541 B542 B543 B544 B545 B546 B547 B548 B549 B550 B551 B552 B553 B554 B555 B556 B557 B558 B559 B560 B561 B562 B563 B564 B565 B566 B567 B568 B569 B570 B571 B572 B573 B574 B575 B576 B577 B578 B579 B580 B581 B582 B583 B584 B585 B586 B587 B588 B589 B590 B591 B592 B593 B594 B595 B596 B597 B598 B599 B600 B601 B602 B603 B604 B605 B606 B607 B608 B609 B610 B611 B612 B613 B614 B615 B616 B617 B618 B619 B620 B621 B622 B623 B624 B625 B626 B627 B628 B629 B630 B631 B632 B633 B634 B635 B636 B637 B638 B639 B640 B641 B642 B643 B644 B645 B646 B647 B648 B649 B650 B651 B652 B653 B654 B655 B656 B657 B658 B659 B660 B661 B662 B663 B664 B665 B666 B667 B668 B669 B670 B671 B672 B673 B674 B675 B676 B677 B678 B679 B680 B681 B682 B683 B684 B685 B686 B687 B688 B689 B690 B691 B692 B693 B694 B695 B696 B697 B698 B699 B700 B701 B702 B703 B704 B705 B706 B707 B708 B709 B710 B711 B712 B713 B714 B715 B716 B717 B718 B719 B720 B721 B722 B723 B724 B725 B726 B727 B728 B729 B730 B731 B732 B733 B734 B735 B736 B737 B738 B739 B740 B741 B742 B743 B744 B745 B746 B747 B748 B749 B750 B751 B752 B753 B754 B755 B756 B757 B758 B759 B760 B761 B762 B763 B764 B765 B766 B767 B768 B769 B770 B771 B772 B773 B774 B775 B776 B777 B778 B779 B780 B781 B782 B783 B784 B785 B786 B787 B788 B789 B790 B791 B792 B793 B794 B795 B796 B797 B798 B799 B800 B801" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="店舗名エラー" error="店舗マスタの一覧にある店舗名を選択してください。" type="list">
       <formula1>店舗マスタ!$A$2:$A$31</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add external (spot) sales section, reorder ranking, rename title
Moves the store ranking table above the 12-month YoY chart, per the
requested page order. Adds an "外販" (external/spot sales) section at
the very bottom: rows where store name is "外販" are split out before
any store aggregation happens, so they never enter store totals,
rankings, or YoY comparisons, and get their own today/YoY/MTD summary
(no forecast, since spot sales don't have a monthly pace to project).
Adds "外販" as a selectable entry in the input template's store
dropdown with a usage note. Also renames the page title from
"多店舗売上ダッシュボード" to "売上ダッシュボード".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155nCVn5tK4kRe72k9sPUbq
</commit_message>
<xml_diff>
--- a/dashboard/templates/日次売上_入力テンプレート.xlsx
+++ b/dashboard/templates/日次売上_入力テンプレート.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -633,6 +633,44 @@
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">　最後の行を選択してコピーし、続きの行に貼り付ければ書式・プルダウンを引き継げます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>【外販（スポット売上）について】</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>・店舗名で「外販」を選ぶと、店舗の売上とは別枠の「外販売上」として記録されます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>・外販の実績は、店舗別の合計・ランキング・前年比などには一切含まれません</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　（ダッシュボード下部に、外販だけの本日・前年同日比・当月累計が別途表示されます）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>・スポットでたまにしか売上が発生しない場合のみ使う想定です。日付・売上金額の入力方法は店舗と同じです。</t>
         </is>
       </c>
     </row>
@@ -731,7 +769,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>外販</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>

</xml_diff>